<commit_message>
Add phase 3B CapEx and executive dashboard tabs
</commit_message>
<xml_diff>
--- a/excel/portfolio_dashboard.xlsx
+++ b/excel/portfolio_dashboard.xlsx
@@ -13,6 +13,8 @@
     <sheet name="Delinquency" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Financials" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Market Comps" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CapEx Projects" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Dashboard" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +72,62 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FF4D4D"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00008000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B2A4A"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00666666"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B2A4A"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -136,7 +194,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -158,11 +216,25 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="001B2A4A"/>
+      </left>
+      <right style="medium">
+        <color rgb="001B2A4A"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B2A4A"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001B2A4A"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -236,6 +308,60 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -17542,4 +17668,1417 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C55A11"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>Total Budgeted</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="26" t="inlineStr">
+        <is>
+          <t>Total Actual</t>
+        </is>
+      </c>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="26" t="inlineStr">
+        <is>
+          <t>Total Variance</t>
+        </is>
+      </c>
+      <c r="H1" s="27" t="n"/>
+      <c r="I1" s="27" t="n"/>
+      <c r="J1" s="26" t="inlineStr">
+        <is>
+          <t>Projects Over Budget</t>
+        </is>
+      </c>
+      <c r="K1" s="27" t="n"/>
+      <c r="L1" s="27" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="27" t="n"/>
+      <c r="B2" s="27" t="n"/>
+      <c r="C2" s="27" t="n"/>
+      <c r="D2" s="27" t="n"/>
+      <c r="E2" s="27" t="n"/>
+      <c r="F2" s="27" t="n"/>
+      <c r="G2" s="27" t="n"/>
+      <c r="H2" s="27" t="n"/>
+      <c r="I2" s="27" t="n"/>
+      <c r="J2" s="27" t="n"/>
+      <c r="K2" s="27" t="n"/>
+      <c r="L2" s="27" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="n">
+        <v>3347000</v>
+      </c>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="28" t="n">
+        <v>3524771.5</v>
+      </c>
+      <c r="E3" s="27" t="n"/>
+      <c r="F3" s="27" t="n"/>
+      <c r="G3" s="29" t="n">
+        <v>177771.5</v>
+      </c>
+      <c r="H3" s="27" t="n"/>
+      <c r="I3" s="27" t="n"/>
+      <c r="J3" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="K3" s="27" t="n"/>
+      <c r="L3" s="27" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="n"/>
+      <c r="B4" s="27" t="n"/>
+      <c r="C4" s="27" t="n"/>
+      <c r="D4" s="27" t="n"/>
+      <c r="E4" s="27" t="n"/>
+      <c r="F4" s="27" t="n"/>
+      <c r="G4" s="27" t="n"/>
+      <c r="H4" s="27" t="n"/>
+      <c r="I4" s="27" t="n"/>
+      <c r="J4" s="27" t="n"/>
+      <c r="K4" s="27" t="n"/>
+      <c r="L4" s="27" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="27" t="n"/>
+      <c r="B5" s="27" t="n"/>
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="27" t="n"/>
+      <c r="F5" s="27" t="n"/>
+      <c r="G5" s="27" t="n"/>
+      <c r="H5" s="27" t="n"/>
+      <c r="I5" s="27" t="n"/>
+      <c r="J5" s="27" t="n"/>
+      <c r="K5" s="27" t="n"/>
+      <c r="L5" s="27" t="n"/>
+    </row>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Property Name</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Asset Type</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Project Type</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Budgeted Cost</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Actual Cost</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Sunrise Meadows</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Entry Road Regrade</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Road Repair</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>45337</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>45442</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>180000</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>187276.61</v>
+      </c>
+      <c r="I9" s="31" t="n">
+        <v>7276.61</v>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="K9" s="13" t="n"/>
+      <c r="L9" s="13" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Desert Palms</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Perimeter Fence Refresh</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Fencing</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>45352</v>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>45463</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>95000</v>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>97479</v>
+      </c>
+      <c r="I10" s="31" t="n">
+        <v>2479</v>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="K10" s="13" t="n"/>
+      <c r="L10" s="13" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Canyon Ridge</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Drainage and Pad Stabilization</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Paving</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>45311</v>
+      </c>
+      <c r="F11" s="14" t="n">
+        <v>45550</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>420000</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>448403.28</v>
+      </c>
+      <c r="I11" s="31" t="n">
+        <v>28403.28</v>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="n"/>
+      <c r="L11" s="13" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Saguaro Estates</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Clubhouse Modernization</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Clubhouse Renovation</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>45392</v>
+      </c>
+      <c r="F12" s="14" t="n">
+        <v>45534</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>260000</v>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>234184.75</v>
+      </c>
+      <c r="I12" s="32" t="n">
+        <v>-25815.25</v>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="K12" s="13" t="n"/>
+      <c r="L12" s="13" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Pinon Pines</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Community-Wide Unit Upgrade Program</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Unit Upgrade</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>45301</v>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>45646</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>780000</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>885148.88</v>
+      </c>
+      <c r="I13" s="31" t="n">
+        <v>105148.88</v>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="K13" s="13" t="n"/>
+      <c r="L13" s="13" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Red Rock Commons</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Domestic Water Loop Upgrade</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Water System</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>45413</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>45596</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>310000</v>
+      </c>
+      <c r="H14" s="19" t="n">
+        <v>302823.2</v>
+      </c>
+      <c r="I14" s="32" t="n">
+        <v>-7176.8</v>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="K14" s="13" t="n"/>
+      <c r="L14" s="13" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Mesa Vista</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Monument Sign Replacement</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Signage</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>45448</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>45498</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>42000</v>
+      </c>
+      <c r="H15" s="19" t="n">
+        <v>43159.45</v>
+      </c>
+      <c r="I15" s="31" t="n">
+        <v>1159.45</v>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="K15" s="13" t="n"/>
+      <c r="L15" s="13" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>ClearBox Storage</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Self-Storage</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>Exterior Lighting and CCTV</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>45334</v>
+      </c>
+      <c r="F16" s="14" t="n">
+        <v>45412</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>165000</v>
+      </c>
+      <c r="H16" s="19" t="n">
+        <v>166499.23</v>
+      </c>
+      <c r="I16" s="31" t="n">
+        <v>1499.23</v>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="K16" s="13" t="n"/>
+      <c r="L16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>SunState Storage</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Self-Storage</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>Drive Aisle Resurfacing</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Paving</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>45371</v>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>45514</v>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>240000</v>
+      </c>
+      <c r="H17" s="19" t="n">
+        <v>267795.95</v>
+      </c>
+      <c r="I17" s="31" t="n">
+        <v>27795.95</v>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="K17" s="13" t="n"/>
+      <c r="L17" s="13" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Desert Vault</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Self-Storage</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>HVAC Retrofit for Climate Units</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>45306</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>45611</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>520000</v>
+      </c>
+      <c r="H18" s="19" t="n">
+        <v>576711.6899999999</v>
+      </c>
+      <c r="I18" s="31" t="n">
+        <v>56711.69</v>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="n"/>
+      <c r="L18" s="13" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Basin Self Storage</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Self-Storage</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>Security Gate and Fence Overhaul</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Fencing</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="n">
+        <v>45383</v>
+      </c>
+      <c r="F19" s="14" t="n">
+        <v>45565</v>
+      </c>
+      <c r="G19" s="19" t="n">
+        <v>210000</v>
+      </c>
+      <c r="H19" s="19" t="n">
+        <v>198494.77</v>
+      </c>
+      <c r="I19" s="32" t="n">
+        <v>-11505.23</v>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="K19" s="13" t="n"/>
+      <c r="L19" s="13" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Summit Storage</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Self-Storage</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>Leasing Office Interior Refresh</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Clubhouse Renovation</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="n">
+        <v>45474</v>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>45595</v>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>125000</v>
+      </c>
+      <c r="H20" s="19" t="n">
+        <v>116794.69</v>
+      </c>
+      <c r="I20" s="32" t="n">
+        <v>-8205.309999999999</v>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="n"/>
+      <c r="L20" s="13" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="D3:F5"/>
+    <mergeCell ref="G1:I2"/>
+    <mergeCell ref="J3:L5"/>
+    <mergeCell ref="J1:L2"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="G3:I5"/>
+    <mergeCell ref="A3:C5"/>
+    <mergeCell ref="D1:F2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C00000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>Executive Portfolio Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>Most Recent Month Performance Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>Total Properties</t>
+        </is>
+      </c>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>Total Units</t>
+        </is>
+      </c>
+      <c r="D3" s="27" t="n"/>
+      <c r="E3" s="35" t="inlineStr">
+        <is>
+          <t>Portfolio Avg Occupancy</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n"/>
+      <c r="G3" s="35" t="inlineStr">
+        <is>
+          <t>Total Monthly NOI</t>
+        </is>
+      </c>
+      <c r="H3" s="27" t="n"/>
+      <c r="I3" s="35" t="inlineStr">
+        <is>
+          <t>Avg Delinquency Rate</t>
+        </is>
+      </c>
+      <c r="J3" s="27" t="n"/>
+      <c r="K3" s="35" t="inlineStr">
+        <is>
+          <t>Total AUM</t>
+        </is>
+      </c>
+      <c r="L3" s="27" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="n"/>
+      <c r="B4" s="27" t="n"/>
+      <c r="C4" s="27" t="n"/>
+      <c r="D4" s="27" t="n"/>
+      <c r="E4" s="27" t="n"/>
+      <c r="F4" s="27" t="n"/>
+      <c r="G4" s="27" t="n"/>
+      <c r="H4" s="27" t="n"/>
+      <c r="I4" s="27" t="n"/>
+      <c r="J4" s="27" t="n"/>
+      <c r="K4" s="27" t="n"/>
+      <c r="L4" s="27" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="B5" s="27" t="n"/>
+      <c r="C5" s="36" t="n">
+        <v>2065</v>
+      </c>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="37" t="n">
+        <v>0.910411622276029</v>
+      </c>
+      <c r="F5" s="27" t="n"/>
+      <c r="G5" s="28" t="n">
+        <v>329033.8900000001</v>
+      </c>
+      <c r="H5" s="27" t="n"/>
+      <c r="I5" s="37" t="n">
+        <v>0.07867780106626204</v>
+      </c>
+      <c r="J5" s="27" t="n"/>
+      <c r="K5" s="28" t="n">
+        <v>111500000</v>
+      </c>
+      <c r="L5" s="27" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="n"/>
+      <c r="B6" s="27" t="n"/>
+      <c r="C6" s="27" t="n"/>
+      <c r="D6" s="27" t="n"/>
+      <c r="E6" s="27" t="n"/>
+      <c r="F6" s="27" t="n"/>
+      <c r="G6" s="27" t="n"/>
+      <c r="H6" s="27" t="n"/>
+      <c r="I6" s="27" t="n"/>
+      <c r="J6" s="27" t="n"/>
+      <c r="K6" s="27" t="n"/>
+      <c r="L6" s="27" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="n"/>
+      <c r="B7" s="27" t="n"/>
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="27" t="n"/>
+      <c r="H7" s="27" t="n"/>
+      <c r="I7" s="27" t="n"/>
+      <c r="J7" s="27" t="n"/>
+      <c r="K7" s="27" t="n"/>
+      <c r="L7" s="27" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="n"/>
+      <c r="B8" s="27" t="n"/>
+      <c r="C8" s="27" t="n"/>
+      <c r="D8" s="27" t="n"/>
+      <c r="E8" s="27" t="n"/>
+      <c r="F8" s="27" t="n"/>
+      <c r="G8" s="27" t="n"/>
+      <c r="H8" s="27" t="n"/>
+      <c r="I8" s="27" t="n"/>
+      <c r="J8" s="27" t="n"/>
+      <c r="K8" s="27" t="n"/>
+      <c r="L8" s="27" t="n"/>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="38" t="inlineStr">
+        <is>
+          <t>Asset Type Comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Self-Storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Avg Occupancy</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>0.9038961038961039</v>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Avg Delinquency</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>0.07907135126575908</v>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>0.07713781404293374</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Total NOI</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n">
+        <v>272752.12</v>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>56281.77</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Avg NOI Margin</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>0.5150428571428571</v>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>0.40846</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Avg Expense Ratio</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>0.4849571428571428</v>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>0.59154</v>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="38" t="inlineStr">
+        <is>
+          <t>Properties Requiring Attention — Most Recent Month</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Property Name</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Asset Type</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Occupancy Rate</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Delinquency Rate</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>NOI</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>NOI Margin</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Risk Label</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Canyon Ridge</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>0.8091</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>0.1567</v>
+      </c>
+      <c r="E22" s="19" t="n">
+        <v>30198.87</v>
+      </c>
+      <c r="F22" s="15" t="n">
+        <v>0.4895</v>
+      </c>
+      <c r="G22" s="39" t="inlineStr">
+        <is>
+          <t>HIGH RISK</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>SunState Storage</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Self-Storage</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>0.9219000000000001</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>0.1268</v>
+      </c>
+      <c r="E23" s="19" t="n">
+        <v>14890.9</v>
+      </c>
+      <c r="F23" s="15" t="n">
+        <v>0.4216</v>
+      </c>
+      <c r="G23" s="40" t="inlineStr">
+        <is>
+          <t>DELINQUENCY RISK</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Mesa Vista</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>0.9304</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>0.1072</v>
+      </c>
+      <c r="E24" s="19" t="n">
+        <v>38999.85</v>
+      </c>
+      <c r="F24" s="15" t="n">
+        <v>0.5009</v>
+      </c>
+      <c r="G24" s="40" t="inlineStr">
+        <is>
+          <t>DELINQUENCY RISK</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Desert Palms</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>0.8947000000000001</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>0.0759</v>
+      </c>
+      <c r="E25" s="19" t="n">
+        <v>30195.35</v>
+      </c>
+      <c r="F25" s="15" t="n">
+        <v>0.5069</v>
+      </c>
+      <c r="G25" s="41" t="inlineStr">
+        <is>
+          <t>OCCUPANCY RISK</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>Pinon Pines</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="n">
+        <v>0.8636</v>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>0.0743</v>
+      </c>
+      <c r="E26" s="19" t="n">
+        <v>24184.75</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>0.4719</v>
+      </c>
+      <c r="G26" s="41" t="inlineStr">
+        <is>
+          <t>OCCUPANCY RISK</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Basin Self Storage</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Self-Storage</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>0.8718</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>0.0672</v>
+      </c>
+      <c r="E27" s="19" t="n">
+        <v>7288.13</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>0.386</v>
+      </c>
+      <c r="G27" s="41" t="inlineStr">
+        <is>
+          <t>OCCUPANCY RISK</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="42" t="inlineStr">
+        <is>
+          <t>This exception report combines occupancy, collections risk, and NOI to help asset managers prioritize follow-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="43" t="inlineStr">
+        <is>
+          <t>Top 5 Properties by NOI Margin</t>
+        </is>
+      </c>
+      <c r="F31" s="43" t="inlineStr">
+        <is>
+          <t>Bottom 5 Properties by NOI Margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Property Name</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Asset Type</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>NOI Margin</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Property Name</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Asset Type</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>NOI Margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="44" t="inlineStr">
+        <is>
+          <t>Saguaro Estates</t>
+        </is>
+      </c>
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C33" s="45" t="n">
+        <v>0.5849</v>
+      </c>
+      <c r="D33" s="13" t="n"/>
+      <c r="E33" s="13" t="n"/>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>Desert Vault</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>Self-Storage</t>
+        </is>
+      </c>
+      <c r="H33" s="15" t="n">
+        <v>0.3258</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="44" t="inlineStr">
+        <is>
+          <t>Red Rock Commons</t>
+        </is>
+      </c>
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C34" s="45" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="D34" s="13" t="n"/>
+      <c r="E34" s="13" t="n"/>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>Basin Self Storage</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>Self-Storage</t>
+        </is>
+      </c>
+      <c r="H34" s="15" t="n">
+        <v>0.386</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="44" t="inlineStr">
+        <is>
+          <t>Sunrise Meadows</t>
+        </is>
+      </c>
+      <c r="B35" s="44" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C35" s="45" t="n">
+        <v>0.5152</v>
+      </c>
+      <c r="D35" s="13" t="n"/>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>SunState Storage</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="inlineStr">
+        <is>
+          <t>Self-Storage</t>
+        </is>
+      </c>
+      <c r="H35" s="15" t="n">
+        <v>0.4216</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="44" t="inlineStr">
+        <is>
+          <t>Desert Palms</t>
+        </is>
+      </c>
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C36" s="45" t="n">
+        <v>0.5069</v>
+      </c>
+      <c r="D36" s="13" t="n"/>
+      <c r="E36" s="13" t="n"/>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Summit Storage</t>
+        </is>
+      </c>
+      <c r="G36" s="13" t="inlineStr">
+        <is>
+          <t>Self-Storage</t>
+        </is>
+      </c>
+      <c r="H36" s="15" t="n">
+        <v>0.4343</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="44" t="inlineStr">
+        <is>
+          <t>Mesa Vista</t>
+        </is>
+      </c>
+      <c r="B37" s="44" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C37" s="45" t="n">
+        <v>0.5009</v>
+      </c>
+      <c r="D37" s="13" t="n"/>
+      <c r="E37" s="13" t="n"/>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>Pinon Pines</t>
+        </is>
+      </c>
+      <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="H37" s="15" t="n">
+        <v>0.4719</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="I3:J4"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="G5:H8"/>
+    <mergeCell ref="I5:J8"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A5:B8"/>
+    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="C3:D4"/>
+    <mergeCell ref="E3:F4"/>
+    <mergeCell ref="K3:L4"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="C5:D8"/>
+    <mergeCell ref="K5:L8"/>
+    <mergeCell ref="E5:F8"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A3:B4"/>
+    <mergeCell ref="G3:H4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add phase 3C acquisition model and insights tabs
</commit_message>
<xml_diff>
--- a/excel/portfolio_dashboard.xlsx
+++ b/excel/portfolio_dashboard.xlsx
@@ -15,6 +15,8 @@
     <sheet name="Market Comps" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="CapEx Projects" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Dashboard" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Acq. Model" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Insights" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,12 +25,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0.00x"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -130,8 +133,36 @@
       <color rgb="00666666"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B2A4A"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -193,6 +224,11 @@
         <fgColor rgb="00A9D18E"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -234,7 +270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -362,6 +398,39 @@
     </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="6" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1135,6 +1204,459 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00006100"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="46" t="inlineStr">
+        <is>
+          <t>Portfolio Findings &amp; Recommended Actions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>Based on 12-month data analysis, January–December 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="62" t="inlineStr">
+        <is>
+          <t>STG-02: Collections Problem, Not a Demand Problem</t>
+        </is>
+      </c>
+      <c r="B4" s="63" t="n"/>
+      <c r="C4" s="63" t="n"/>
+      <c r="D4" s="63" t="n"/>
+      <c r="E4" s="63" t="n"/>
+      <c r="F4" s="63" t="n"/>
+      <c r="G4" s="63" t="n"/>
+      <c r="H4" s="63" t="n"/>
+      <c r="I4" s="63" t="n"/>
+      <c r="J4" s="63" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="64" t="inlineStr">
+        <is>
+          <t>SunState Storage | Self-Storage | Good occupancy but delinquency rising from approximately 7% to 13%</t>
+        </is>
+      </c>
+      <c r="B5" s="63" t="n"/>
+      <c r="C5" s="63" t="n"/>
+      <c r="D5" s="63" t="n"/>
+      <c r="E5" s="63" t="n"/>
+      <c r="F5" s="63" t="n"/>
+      <c r="G5" s="63" t="n"/>
+      <c r="H5" s="63" t="n"/>
+      <c r="I5" s="63" t="n"/>
+      <c r="J5" s="63" t="n"/>
+    </row>
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="65" t="inlineStr">
+        <is>
+          <t>Data shows: STG-02 maintained generally healthy occupancy, which suggests demand is not the primary issue. The bigger concern is the upward delinquency trend, meaning revenue leakage is coming from collections rather than lack of tenants.</t>
+        </is>
+      </c>
+      <c r="B6" s="63" t="n"/>
+      <c r="C6" s="63" t="n"/>
+      <c r="D6" s="63" t="n"/>
+      <c r="E6" s="63" t="n"/>
+      <c r="F6" s="63" t="n"/>
+      <c r="G6" s="63" t="n"/>
+      <c r="H6" s="63" t="n"/>
+      <c r="I6" s="63" t="n"/>
+      <c r="J6" s="63" t="n"/>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="66" t="inlineStr">
+        <is>
+          <t>Recommended action: Review aged receivables, late-fee enforcement, payment reminders, and property-level collection workflows. The asset management team should work with property operations to reduce delinquency before it impacts NOI further.</t>
+        </is>
+      </c>
+      <c r="B7" s="63" t="n"/>
+      <c r="C7" s="63" t="n"/>
+      <c r="D7" s="63" t="n"/>
+      <c r="E7" s="63" t="n"/>
+      <c r="F7" s="63" t="n"/>
+      <c r="G7" s="63" t="n"/>
+      <c r="H7" s="63" t="n"/>
+      <c r="I7" s="63" t="n"/>
+      <c r="J7" s="63" t="n"/>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="62" t="inlineStr">
+        <is>
+          <t>MHC-03: Dual-Flag Asset Requiring Immediate Operational Review</t>
+        </is>
+      </c>
+      <c r="B9" s="63" t="n"/>
+      <c r="C9" s="63" t="n"/>
+      <c r="D9" s="63" t="n"/>
+      <c r="E9" s="63" t="n"/>
+      <c r="F9" s="63" t="n"/>
+      <c r="G9" s="63" t="n"/>
+      <c r="H9" s="63" t="n"/>
+      <c r="I9" s="63" t="n"/>
+      <c r="J9" s="63" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="64" t="inlineStr">
+        <is>
+          <t>Canyon Ridge | MHC | Low occupancy around 78–83% and high delinquency around 12–16%</t>
+        </is>
+      </c>
+      <c r="B10" s="63" t="n"/>
+      <c r="C10" s="63" t="n"/>
+      <c r="D10" s="63" t="n"/>
+      <c r="E10" s="63" t="n"/>
+      <c r="F10" s="63" t="n"/>
+      <c r="G10" s="63" t="n"/>
+      <c r="H10" s="63" t="n"/>
+      <c r="I10" s="63" t="n"/>
+      <c r="J10" s="63" t="n"/>
+    </row>
+    <row r="11" ht="55" customHeight="1">
+      <c r="A11" s="65" t="inlineStr">
+        <is>
+          <t>Data shows: MHC-03 is the weakest risk profile in the portfolio because it has both demand weakness and collections risk. This combination can pressure revenue, NOI, and investor reporting.</t>
+        </is>
+      </c>
+      <c r="B11" s="63" t="n"/>
+      <c r="C11" s="63" t="n"/>
+      <c r="D11" s="63" t="n"/>
+      <c r="E11" s="63" t="n"/>
+      <c r="F11" s="63" t="n"/>
+      <c r="G11" s="63" t="n"/>
+      <c r="H11" s="63" t="n"/>
+      <c r="I11" s="63" t="n"/>
+      <c r="J11" s="63" t="n"/>
+    </row>
+    <row r="12" ht="55" customHeight="1">
+      <c r="A12" s="66" t="inlineStr">
+        <is>
+          <t>Recommended action: Prioritize an operational review covering leasing activity, local market positioning, rent levels, resident retention, and collections. This property should be included in weekly asset management follow-up until both occupancy and delinquency stabilize.</t>
+        </is>
+      </c>
+      <c r="B12" s="63" t="n"/>
+      <c r="C12" s="63" t="n"/>
+      <c r="D12" s="63" t="n"/>
+      <c r="E12" s="63" t="n"/>
+      <c r="F12" s="63" t="n"/>
+      <c r="G12" s="63" t="n"/>
+      <c r="H12" s="63" t="n"/>
+      <c r="I12" s="63" t="n"/>
+      <c r="J12" s="63" t="n"/>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="62" t="inlineStr">
+        <is>
+          <t>MHC-04: Portfolio Benchmark — Operational Best Practices Template</t>
+        </is>
+      </c>
+      <c r="B14" s="63" t="n"/>
+      <c r="C14" s="63" t="n"/>
+      <c r="D14" s="63" t="n"/>
+      <c r="E14" s="63" t="n"/>
+      <c r="F14" s="63" t="n"/>
+      <c r="G14" s="63" t="n"/>
+      <c r="H14" s="63" t="n"/>
+      <c r="I14" s="63" t="n"/>
+      <c r="J14" s="63" t="n"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="64" t="inlineStr">
+        <is>
+          <t>Saguaro Estates | MHC | High occupancy, low delinquency, strong NOI margin</t>
+        </is>
+      </c>
+      <c r="B15" s="63" t="n"/>
+      <c r="C15" s="63" t="n"/>
+      <c r="D15" s="63" t="n"/>
+      <c r="E15" s="63" t="n"/>
+      <c r="F15" s="63" t="n"/>
+      <c r="G15" s="63" t="n"/>
+      <c r="H15" s="63" t="n"/>
+      <c r="I15" s="63" t="n"/>
+      <c r="J15" s="63" t="n"/>
+    </row>
+    <row r="16" ht="55" customHeight="1">
+      <c r="A16" s="65" t="inlineStr">
+        <is>
+          <t>Data shows: MHC-04 performs like a benchmark asset, with high occupancy, low delinquency, and strong profitability. This indicates strong property-level execution and stable resident demand.</t>
+        </is>
+      </c>
+      <c r="B16" s="63" t="n"/>
+      <c r="C16" s="63" t="n"/>
+      <c r="D16" s="63" t="n"/>
+      <c r="E16" s="63" t="n"/>
+      <c r="F16" s="63" t="n"/>
+      <c r="G16" s="63" t="n"/>
+      <c r="H16" s="63" t="n"/>
+      <c r="I16" s="63" t="n"/>
+      <c r="J16" s="63" t="n"/>
+    </row>
+    <row r="17" ht="55" customHeight="1">
+      <c r="A17" s="66" t="inlineStr">
+        <is>
+          <t>Recommended action: Use MHC-04 as an internal operating benchmark. Compare staffing, collections process, leasing practices, resident communication, and expense controls against weaker MHC assets.</t>
+        </is>
+      </c>
+      <c r="B17" s="63" t="n"/>
+      <c r="C17" s="63" t="n"/>
+      <c r="D17" s="63" t="n"/>
+      <c r="E17" s="63" t="n"/>
+      <c r="F17" s="63" t="n"/>
+      <c r="G17" s="63" t="n"/>
+      <c r="H17" s="63" t="n"/>
+      <c r="I17" s="63" t="n"/>
+      <c r="J17" s="63" t="n"/>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="62" t="inlineStr">
+        <is>
+          <t>MHC-05: Value-Add Play — Track Against Pro Forma Monthly</t>
+        </is>
+      </c>
+      <c r="B19" s="63" t="n"/>
+      <c r="C19" s="63" t="n"/>
+      <c r="D19" s="63" t="n"/>
+      <c r="E19" s="63" t="n"/>
+      <c r="F19" s="63" t="n"/>
+      <c r="G19" s="63" t="n"/>
+      <c r="H19" s="63" t="n"/>
+      <c r="I19" s="63" t="n"/>
+      <c r="J19" s="63" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="64" t="inlineStr">
+        <is>
+          <t>Pinon Pines | MHC | Occupancy improves from roughly 81% to 89% over the year</t>
+        </is>
+      </c>
+      <c r="B20" s="63" t="n"/>
+      <c r="C20" s="63" t="n"/>
+      <c r="D20" s="63" t="n"/>
+      <c r="E20" s="63" t="n"/>
+      <c r="F20" s="63" t="n"/>
+      <c r="G20" s="63" t="n"/>
+      <c r="H20" s="63" t="n"/>
+      <c r="I20" s="63" t="n"/>
+      <c r="J20" s="63" t="n"/>
+    </row>
+    <row r="21" ht="55" customHeight="1">
+      <c r="A21" s="65" t="inlineStr">
+        <is>
+          <t>Data shows: MHC-05 shows a positive value-add trend with improving occupancy, but it has not yet reached stabilized performance. The asset has rent upside and operational upside, making it a good candidate for active tracking.</t>
+        </is>
+      </c>
+      <c r="B21" s="63" t="n"/>
+      <c r="C21" s="63" t="n"/>
+      <c r="D21" s="63" t="n"/>
+      <c r="E21" s="63" t="n"/>
+      <c r="F21" s="63" t="n"/>
+      <c r="G21" s="63" t="n"/>
+      <c r="H21" s="63" t="n"/>
+      <c r="I21" s="63" t="n"/>
+      <c r="J21" s="63" t="n"/>
+    </row>
+    <row r="22" ht="55" customHeight="1">
+      <c r="A22" s="66" t="inlineStr">
+        <is>
+          <t>Recommended action: Track MHC-05 monthly against the acquisition pro forma, especially occupancy, rent growth, CapEx spend, and NOI margin. Management should confirm that renovation dollars are converting into occupancy gains and stronger cash flow.</t>
+        </is>
+      </c>
+      <c r="B22" s="63" t="n"/>
+      <c r="C22" s="63" t="n"/>
+      <c r="D22" s="63" t="n"/>
+      <c r="E22" s="63" t="n"/>
+      <c r="F22" s="63" t="n"/>
+      <c r="G22" s="63" t="n"/>
+      <c r="H22" s="63" t="n"/>
+      <c r="I22" s="63" t="n"/>
+      <c r="J22" s="63" t="n"/>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="62" t="inlineStr">
+        <is>
+          <t>STG-03: Expense Ratio Drag — NOI Underperformance Despite Adequate Occupancy</t>
+        </is>
+      </c>
+      <c r="B24" s="63" t="n"/>
+      <c r="C24" s="63" t="n"/>
+      <c r="D24" s="63" t="n"/>
+      <c r="E24" s="63" t="n"/>
+      <c r="F24" s="63" t="n"/>
+      <c r="G24" s="63" t="n"/>
+      <c r="H24" s="63" t="n"/>
+      <c r="I24" s="63" t="n"/>
+      <c r="J24" s="63" t="n"/>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="64" t="inlineStr">
+        <is>
+          <t>Desert Vault | Self-Storage | Expense ratio around 62–68%</t>
+        </is>
+      </c>
+      <c r="B25" s="63" t="n"/>
+      <c r="C25" s="63" t="n"/>
+      <c r="D25" s="63" t="n"/>
+      <c r="E25" s="63" t="n"/>
+      <c r="F25" s="63" t="n"/>
+      <c r="G25" s="63" t="n"/>
+      <c r="H25" s="63" t="n"/>
+      <c r="I25" s="63" t="n"/>
+      <c r="J25" s="63" t="n"/>
+    </row>
+    <row r="26" ht="55" customHeight="1">
+      <c r="A26" s="65" t="inlineStr">
+        <is>
+          <t>Data shows: STG-03 does not appear to be purely an occupancy problem. The high expense ratio is reducing NOI margin and making the property less profitable than it should be.</t>
+        </is>
+      </c>
+      <c r="B26" s="63" t="n"/>
+      <c r="C26" s="63" t="n"/>
+      <c r="D26" s="63" t="n"/>
+      <c r="E26" s="63" t="n"/>
+      <c r="F26" s="63" t="n"/>
+      <c r="G26" s="63" t="n"/>
+      <c r="H26" s="63" t="n"/>
+      <c r="I26" s="63" t="n"/>
+      <c r="J26" s="63" t="n"/>
+    </row>
+    <row r="27" ht="55" customHeight="1">
+      <c r="A27" s="66" t="inlineStr">
+        <is>
+          <t>Recommended action: Review controllable expenses such as repairs, payroll, utilities, vendor contracts, insurance, and recurring maintenance. The finance and asset management teams should isolate which expense categories are driving margin compression.</t>
+        </is>
+      </c>
+      <c r="B27" s="63" t="n"/>
+      <c r="C27" s="63" t="n"/>
+      <c r="D27" s="63" t="n"/>
+      <c r="E27" s="63" t="n"/>
+      <c r="F27" s="63" t="n"/>
+      <c r="G27" s="63" t="n"/>
+      <c r="H27" s="63" t="n"/>
+      <c r="I27" s="63" t="n"/>
+      <c r="J27" s="63" t="n"/>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="62" t="inlineStr">
+        <is>
+          <t>MHC-07: Early Warning — Delinquency Trend Requires Collections Intervention Before It Escalates</t>
+        </is>
+      </c>
+      <c r="B29" s="63" t="n"/>
+      <c r="C29" s="63" t="n"/>
+      <c r="D29" s="63" t="n"/>
+      <c r="E29" s="63" t="n"/>
+      <c r="F29" s="63" t="n"/>
+      <c r="G29" s="63" t="n"/>
+      <c r="H29" s="63" t="n"/>
+      <c r="I29" s="63" t="n"/>
+      <c r="J29" s="63" t="n"/>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="64" t="inlineStr">
+        <is>
+          <t>Mesa Vista | MHC | High occupancy but delinquency rising from approximately 5% to 11%</t>
+        </is>
+      </c>
+      <c r="B30" s="63" t="n"/>
+      <c r="C30" s="63" t="n"/>
+      <c r="D30" s="63" t="n"/>
+      <c r="E30" s="63" t="n"/>
+      <c r="F30" s="63" t="n"/>
+      <c r="G30" s="63" t="n"/>
+      <c r="H30" s="63" t="n"/>
+      <c r="I30" s="63" t="n"/>
+      <c r="J30" s="63" t="n"/>
+    </row>
+    <row r="31" ht="55" customHeight="1">
+      <c r="A31" s="65" t="inlineStr">
+        <is>
+          <t>Data shows: MHC-07 still has strong occupancy, but the delinquency trend is moving in the wrong direction. This is an early warning sign because the property looks healthy from an occupancy view but has growing collection risk.</t>
+        </is>
+      </c>
+      <c r="B31" s="63" t="n"/>
+      <c r="C31" s="63" t="n"/>
+      <c r="D31" s="63" t="n"/>
+      <c r="E31" s="63" t="n"/>
+      <c r="F31" s="63" t="n"/>
+      <c r="G31" s="63" t="n"/>
+      <c r="H31" s="63" t="n"/>
+      <c r="I31" s="63" t="n"/>
+      <c r="J31" s="63" t="n"/>
+    </row>
+    <row r="32" ht="55" customHeight="1">
+      <c r="A32" s="66" t="inlineStr">
+        <is>
+          <t>Recommended action: Intervene before the issue becomes critical by reviewing tenant aging buckets, payment plan usage, late-fee timing, and property manager follow-up. This should be treated as a collections process issue before assuming a demand issue.</t>
+        </is>
+      </c>
+      <c r="B32" s="63" t="n"/>
+      <c r="C32" s="63" t="n"/>
+      <c r="D32" s="63" t="n"/>
+      <c r="E32" s="63" t="n"/>
+      <c r="F32" s="63" t="n"/>
+      <c r="G32" s="63" t="n"/>
+      <c r="H32" s="63" t="n"/>
+      <c r="I32" s="63" t="n"/>
+      <c r="J32" s="63" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="26">
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A32:J32"/>
+    <mergeCell ref="A14:J14"/>
+    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A10:J10"/>
+    <mergeCell ref="A19:J19"/>
+    <mergeCell ref="A31:J31"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A30:J30"/>
+    <mergeCell ref="A15:J15"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A25:J25"/>
+    <mergeCell ref="A27:J27"/>
+    <mergeCell ref="A21:J21"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -19081,4 +19603,808 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FFD700"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="46" t="inlineStr">
+        <is>
+          <t>Acquisition Underwriting — MHC-05 Pinon Pines</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="47" t="inlineStr">
+        <is>
+          <t>Underwriting Assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="48" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="B3" s="49" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="50" t="inlineStr">
+        <is>
+          <t>Total Units</t>
+        </is>
+      </c>
+      <c r="B4" s="51" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="50" t="inlineStr">
+        <is>
+          <t>Current Occupancy</t>
+        </is>
+      </c>
+      <c r="B5" s="52" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="50" t="inlineStr">
+        <is>
+          <t>Stabilized Occupancy Target</t>
+        </is>
+      </c>
+      <c r="B6" s="52" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="50" t="inlineStr">
+        <is>
+          <t>Current Avg Monthly Rent per Lot</t>
+        </is>
+      </c>
+      <c r="B7" s="53" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="50" t="inlineStr">
+        <is>
+          <t>Market Avg Rent</t>
+        </is>
+      </c>
+      <c r="B8" s="53" t="n">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="50" t="inlineStr">
+        <is>
+          <t>Year 1 Rent Growth</t>
+        </is>
+      </c>
+      <c r="B9" s="52" t="n">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="50" t="inlineStr">
+        <is>
+          <t>Years 2-5 Rent Growth</t>
+        </is>
+      </c>
+      <c r="B10" s="52" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="50" t="inlineStr">
+        <is>
+          <t>Operating Expense Ratio Year 1</t>
+        </is>
+      </c>
+      <c r="B11" s="52" t="n">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="50" t="inlineStr">
+        <is>
+          <t>Expense Ratio Improvement</t>
+        </is>
+      </c>
+      <c r="B12" s="52" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="50" t="inlineStr">
+        <is>
+          <t>Renovation CapEx Year 1</t>
+        </is>
+      </c>
+      <c r="B13" s="53" t="n">
+        <v>380000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="50" t="inlineStr">
+        <is>
+          <t>Exit Cap Rate</t>
+        </is>
+      </c>
+      <c r="B14" s="54" t="n">
+        <v>0.0625</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="50" t="inlineStr">
+        <is>
+          <t>Loan Amount</t>
+        </is>
+      </c>
+      <c r="B15" s="53" t="n">
+        <v>2730000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="50" t="inlineStr">
+        <is>
+          <t>Interest Rate</t>
+        </is>
+      </c>
+      <c r="B16" s="52" t="n">
+        <v>0.068</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="50" t="inlineStr">
+        <is>
+          <t>Loan Term</t>
+        </is>
+      </c>
+      <c r="B17" s="51" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="50" t="inlineStr">
+        <is>
+          <t>Acquisition Costs</t>
+        </is>
+      </c>
+      <c r="B18" s="52" t="n">
+        <v>0.025</v>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="47" t="inlineStr">
+        <is>
+          <t>5-Year Operating Pro Forma</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="50" t="inlineStr">
+        <is>
+          <t>Occupied Units</t>
+        </is>
+      </c>
+      <c r="B24" s="55" t="n">
+        <v>74</v>
+      </c>
+      <c r="C24" s="55" t="n">
+        <v>76</v>
+      </c>
+      <c r="D24" s="55" t="n">
+        <v>78</v>
+      </c>
+      <c r="E24" s="55" t="n">
+        <v>80</v>
+      </c>
+      <c r="F24" s="55" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="50" t="inlineStr">
+        <is>
+          <t>Occupancy Rate</t>
+        </is>
+      </c>
+      <c r="B25" s="56" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="C25" s="56" t="n">
+        <v>0.865</v>
+      </c>
+      <c r="D25" s="56" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="E25" s="56" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="F25" s="56" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="50" t="inlineStr">
+        <is>
+          <t>Avg Monthly Rent</t>
+        </is>
+      </c>
+      <c r="B26" s="57" t="n">
+        <v>752.4</v>
+      </c>
+      <c r="C26" s="57" t="n">
+        <v>774.972</v>
+      </c>
+      <c r="D26" s="57" t="n">
+        <v>798.2211600000001</v>
+      </c>
+      <c r="E26" s="57" t="n">
+        <v>822.1677948</v>
+      </c>
+      <c r="F26" s="57" t="n">
+        <v>846.8328286440001</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="50" t="inlineStr">
+        <is>
+          <t>Gross Potential Rent Annual</t>
+        </is>
+      </c>
+      <c r="B27" s="57" t="n">
+        <v>794534.3999999999</v>
+      </c>
+      <c r="C27" s="57" t="n">
+        <v>818370.4319999999</v>
+      </c>
+      <c r="D27" s="57" t="n">
+        <v>842921.54496</v>
+      </c>
+      <c r="E27" s="57" t="n">
+        <v>868209.1913088</v>
+      </c>
+      <c r="F27" s="57" t="n">
+        <v>894255.467048064</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="50" t="inlineStr">
+        <is>
+          <t>Vacancy Loss</t>
+        </is>
+      </c>
+      <c r="B28" s="57" t="n">
+        <v>127125.504</v>
+      </c>
+      <c r="C28" s="57" t="n">
+        <v>110480.00832</v>
+      </c>
+      <c r="D28" s="57" t="n">
+        <v>92721.36994559999</v>
+      </c>
+      <c r="E28" s="57" t="n">
+        <v>78138.82721779197</v>
+      </c>
+      <c r="F28" s="57" t="n">
+        <v>62597.88269336444</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="50" t="inlineStr">
+        <is>
+          <t>Effective Gross Income</t>
+        </is>
+      </c>
+      <c r="B29" s="57" t="n">
+        <v>667408.8959999999</v>
+      </c>
+      <c r="C29" s="57" t="n">
+        <v>707890.4236799999</v>
+      </c>
+      <c r="D29" s="57" t="n">
+        <v>750200.1750143999</v>
+      </c>
+      <c r="E29" s="57" t="n">
+        <v>790070.3640910081</v>
+      </c>
+      <c r="F29" s="57" t="n">
+        <v>831657.5843546996</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="50" t="inlineStr">
+        <is>
+          <t>Operating Expenses</t>
+        </is>
+      </c>
+      <c r="B30" s="57" t="n">
+        <v>320356.27008</v>
+      </c>
+      <c r="C30" s="57" t="n">
+        <v>332708.4991295999</v>
+      </c>
+      <c r="D30" s="57" t="n">
+        <v>345092.080506624</v>
+      </c>
+      <c r="E30" s="57" t="n">
+        <v>355531.6638409536</v>
+      </c>
+      <c r="F30" s="57" t="n">
+        <v>365929.3371160678</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="50" t="inlineStr">
+        <is>
+          <t>NOI</t>
+        </is>
+      </c>
+      <c r="B31" s="57" t="n">
+        <v>347052.62592</v>
+      </c>
+      <c r="C31" s="57" t="n">
+        <v>375181.9245503999</v>
+      </c>
+      <c r="D31" s="57" t="n">
+        <v>405108.094507776</v>
+      </c>
+      <c r="E31" s="57" t="n">
+        <v>434538.7002500545</v>
+      </c>
+      <c r="F31" s="57" t="n">
+        <v>465728.2472386318</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="50" t="inlineStr">
+        <is>
+          <t>NOI Margin %</t>
+        </is>
+      </c>
+      <c r="B32" s="56" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="C32" s="56" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="D32" s="56" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="E32" s="56" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F32" s="56" t="n">
+        <v>0.5599999999999999</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="50" t="inlineStr">
+        <is>
+          <t>Debt Service Annual P&amp;I</t>
+        </is>
+      </c>
+      <c r="B33" s="57" t="n">
+        <v>385104.9324103267</v>
+      </c>
+      <c r="C33" s="57" t="n">
+        <v>385104.9324103267</v>
+      </c>
+      <c r="D33" s="57" t="n">
+        <v>385104.9324103267</v>
+      </c>
+      <c r="E33" s="57" t="n">
+        <v>385104.9324103267</v>
+      </c>
+      <c r="F33" s="57" t="n">
+        <v>385104.9324103267</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="50" t="inlineStr">
+        <is>
+          <t>Net Cash Flow After Debt</t>
+        </is>
+      </c>
+      <c r="B34" s="57" t="n">
+        <v>-38052.30649032677</v>
+      </c>
+      <c r="C34" s="57" t="n">
+        <v>-9923.007859926787</v>
+      </c>
+      <c r="D34" s="57" t="n">
+        <v>20003.16209744924</v>
+      </c>
+      <c r="E34" s="57" t="n">
+        <v>49433.76783972775</v>
+      </c>
+      <c r="F34" s="57" t="n">
+        <v>80623.31482830504</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="50" t="inlineStr">
+        <is>
+          <t>Cash-on-Cash Return</t>
+        </is>
+      </c>
+      <c r="B35" s="56" t="n">
+        <v>-0.01946409539147149</v>
+      </c>
+      <c r="C35" s="56" t="n">
+        <v>-0.005075707345231093</v>
+      </c>
+      <c r="D35" s="56" t="n">
+        <v>0.0102317964692835</v>
+      </c>
+      <c r="E35" s="56" t="n">
+        <v>0.0252858147517789</v>
+      </c>
+      <c r="F35" s="56" t="n">
+        <v>0.0412395472267545</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="50" t="inlineStr">
+        <is>
+          <t>Cumulative Cash Flow</t>
+        </is>
+      </c>
+      <c r="B36" s="57" t="n">
+        <v>-38052.30649032677</v>
+      </c>
+      <c r="C36" s="57" t="n">
+        <v>-47975.31435025355</v>
+      </c>
+      <c r="D36" s="57" t="n">
+        <v>-27972.15225280431</v>
+      </c>
+      <c r="E36" s="57" t="n">
+        <v>21461.61558692344</v>
+      </c>
+      <c r="F36" s="57" t="n">
+        <v>102084.9304152285</v>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="58" t="inlineStr">
+        <is>
+          <t>Exit Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="50" t="inlineStr">
+        <is>
+          <t>Year 5 Exit Value</t>
+        </is>
+      </c>
+      <c r="B40" s="57" t="n">
+        <v>7451651.955818108</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="50" t="inlineStr">
+        <is>
+          <t>Remaining Loan Balance after 5 years</t>
+        </is>
+      </c>
+      <c r="B41" s="57" t="n">
+        <v>1587498.069811833</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="50" t="inlineStr">
+        <is>
+          <t>Net Proceeds</t>
+        </is>
+      </c>
+      <c r="B42" s="57" t="n">
+        <v>5864153.886006275</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="50" t="inlineStr">
+        <is>
+          <t>Cumulative Cash Flow</t>
+        </is>
+      </c>
+      <c r="B43" s="57" t="n">
+        <v>102084.9304152285</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="50" t="inlineStr">
+        <is>
+          <t>Total Return</t>
+        </is>
+      </c>
+      <c r="B44" s="57" t="n">
+        <v>5966238.816421503</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="50" t="inlineStr">
+        <is>
+          <t>Initial Equity</t>
+        </is>
+      </c>
+      <c r="B45" s="57" t="n">
+        <v>1955000</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="50" t="inlineStr">
+        <is>
+          <t>Equity Multiple</t>
+        </is>
+      </c>
+      <c r="B46" s="59" t="n">
+        <v>3.051784560829413</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="50" t="inlineStr">
+        <is>
+          <t>IRR</t>
+        </is>
+      </c>
+      <c r="B47" s="56" t="n">
+        <v>0.2483095921905548</v>
+      </c>
+    </row>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="58" t="inlineStr">
+        <is>
+          <t>IRR Sensitivity — Exit Cap Rate vs Year 5 NOI Scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>Exit Cap Rate</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>−5%</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>+10%</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="60" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="B52" s="61" t="n">
+        <v>0.2721047563746169</v>
+      </c>
+      <c r="C52" s="61" t="n">
+        <v>0.2880719075812196</v>
+      </c>
+      <c r="D52" s="61" t="n">
+        <v>0.2880719075812196</v>
+      </c>
+      <c r="E52" s="61" t="n">
+        <v>0.3032849461413913</v>
+      </c>
+      <c r="F52" s="61" t="n">
+        <v>0.3178196192521103</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="60" t="n">
+        <v>0.0575</v>
+      </c>
+      <c r="B53" s="61" t="n">
+        <v>0.2582824296655034</v>
+      </c>
+      <c r="C53" s="61" t="n">
+        <v>0.2742332082475913</v>
+      </c>
+      <c r="D53" s="61" t="n">
+        <v>0.2742332082475913</v>
+      </c>
+      <c r="E53" s="61" t="n">
+        <v>0.2894235400893012</v>
+      </c>
+      <c r="F53" s="61" t="n">
+        <v>0.3039304914532881</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="60" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="B54" s="61" t="n">
+        <v>0.2450556241915656</v>
+      </c>
+      <c r="C54" s="61" t="n">
+        <v>0.2609973815794902</v>
+      </c>
+      <c r="D54" s="61" t="n">
+        <v>0.2609973815794902</v>
+      </c>
+      <c r="E54" s="61" t="n">
+        <v>0.2761718810378718</v>
+      </c>
+      <c r="F54" s="61" t="n">
+        <v>0.2906575807022166</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="60" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="B55" s="61" t="n">
+        <v>0.2323699848946241</v>
+      </c>
+      <c r="C55" s="61" t="n">
+        <v>0.2483095921905548</v>
+      </c>
+      <c r="D55" s="61" t="n">
+        <v>0.2483095921905548</v>
+      </c>
+      <c r="E55" s="61" t="n">
+        <v>0.2634746628613108</v>
+      </c>
+      <c r="F55" s="61" t="n">
+        <v>0.2779451207263591</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="60" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="B56" s="61" t="n">
+        <v>0.22017788947152</v>
+      </c>
+      <c r="C56" s="61" t="n">
+        <v>0.2361218059578299</v>
+      </c>
+      <c r="D56" s="61" t="n">
+        <v>0.2361218059578299</v>
+      </c>
+      <c r="E56" s="61" t="n">
+        <v>0.2512834462014333</v>
+      </c>
+      <c r="F56" s="61" t="n">
+        <v>0.2657442748722254</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="60" t="n">
+        <v>0.0675</v>
+      </c>
+      <c r="B57" s="61" t="n">
+        <v>0.2084373850784495</v>
+      </c>
+      <c r="C57" s="61" t="n">
+        <v>0.2243917162125861</v>
+      </c>
+      <c r="D57" s="61" t="n">
+        <v>0.2243917162125861</v>
+      </c>
+      <c r="E57" s="61" t="n">
+        <v>0.2395555745201499</v>
+      </c>
+      <c r="F57" s="61" t="n">
+        <v>0.2540120423711922</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="60" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="B58" s="61" t="n">
+        <v>0.197111325171002</v>
+      </c>
+      <c r="C58" s="61" t="n">
+        <v>0.2130818720811583</v>
+      </c>
+      <c r="D58" s="61" t="n">
+        <v>0.2130818720811583</v>
+      </c>
+      <c r="E58" s="61" t="n">
+        <v>0.2282532942369244</v>
+      </c>
+      <c r="F58" s="61" t="n">
+        <v>0.2427103705538361</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add final project documentation
</commit_message>
<xml_diff>
--- a/excel/portfolio_dashboard.xlsx
+++ b/excel/portfolio_dashboard.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.00x"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -112,6 +112,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001B2A4A"/>
       <sz val="12"/>
@@ -129,12 +135,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00666666"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001B2A4A"/>
       <sz val="16"/>
@@ -144,11 +144,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -270,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -382,17 +377,20 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -406,36 +404,59 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="6" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="6" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -1227,7 +1248,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="46" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>Portfolio Findings &amp; Recommended Actions</t>
         </is>
@@ -1241,388 +1262,388 @@
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="62" t="inlineStr">
+      <c r="A4" s="63" t="inlineStr">
         <is>
           <t>STG-02: Collections Problem, Not a Demand Problem</t>
         </is>
       </c>
-      <c r="B4" s="63" t="n"/>
-      <c r="C4" s="63" t="n"/>
-      <c r="D4" s="63" t="n"/>
-      <c r="E4" s="63" t="n"/>
-      <c r="F4" s="63" t="n"/>
-      <c r="G4" s="63" t="n"/>
-      <c r="H4" s="63" t="n"/>
-      <c r="I4" s="63" t="n"/>
-      <c r="J4" s="63" t="n"/>
+      <c r="B4" s="64" t="n"/>
+      <c r="C4" s="64" t="n"/>
+      <c r="D4" s="64" t="n"/>
+      <c r="E4" s="64" t="n"/>
+      <c r="F4" s="64" t="n"/>
+      <c r="G4" s="64" t="n"/>
+      <c r="H4" s="64" t="n"/>
+      <c r="I4" s="64" t="n"/>
+      <c r="J4" s="64" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="64" t="inlineStr">
+      <c r="A5" s="65" t="inlineStr">
         <is>
           <t>SunState Storage | Self-Storage | Good occupancy but delinquency rising from approximately 7% to 13%</t>
         </is>
       </c>
-      <c r="B5" s="63" t="n"/>
-      <c r="C5" s="63" t="n"/>
-      <c r="D5" s="63" t="n"/>
-      <c r="E5" s="63" t="n"/>
-      <c r="F5" s="63" t="n"/>
-      <c r="G5" s="63" t="n"/>
-      <c r="H5" s="63" t="n"/>
-      <c r="I5" s="63" t="n"/>
-      <c r="J5" s="63" t="n"/>
+      <c r="B5" s="64" t="n"/>
+      <c r="C5" s="64" t="n"/>
+      <c r="D5" s="64" t="n"/>
+      <c r="E5" s="64" t="n"/>
+      <c r="F5" s="64" t="n"/>
+      <c r="G5" s="64" t="n"/>
+      <c r="H5" s="64" t="n"/>
+      <c r="I5" s="64" t="n"/>
+      <c r="J5" s="64" t="n"/>
     </row>
     <row r="6" ht="55" customHeight="1">
-      <c r="A6" s="65" t="inlineStr">
+      <c r="A6" s="66" t="inlineStr">
         <is>
           <t>Data shows: STG-02 maintained generally healthy occupancy, which suggests demand is not the primary issue. The bigger concern is the upward delinquency trend, meaning revenue leakage is coming from collections rather than lack of tenants.</t>
         </is>
       </c>
-      <c r="B6" s="63" t="n"/>
-      <c r="C6" s="63" t="n"/>
-      <c r="D6" s="63" t="n"/>
-      <c r="E6" s="63" t="n"/>
-      <c r="F6" s="63" t="n"/>
-      <c r="G6" s="63" t="n"/>
-      <c r="H6" s="63" t="n"/>
-      <c r="I6" s="63" t="n"/>
-      <c r="J6" s="63" t="n"/>
+      <c r="B6" s="64" t="n"/>
+      <c r="C6" s="64" t="n"/>
+      <c r="D6" s="64" t="n"/>
+      <c r="E6" s="64" t="n"/>
+      <c r="F6" s="64" t="n"/>
+      <c r="G6" s="64" t="n"/>
+      <c r="H6" s="64" t="n"/>
+      <c r="I6" s="64" t="n"/>
+      <c r="J6" s="64" t="n"/>
     </row>
     <row r="7" ht="55" customHeight="1">
-      <c r="A7" s="66" t="inlineStr">
+      <c r="A7" s="67" t="inlineStr">
         <is>
           <t>Recommended action: Review aged receivables, late-fee enforcement, payment reminders, and property-level collection workflows. The asset management team should work with property operations to reduce delinquency before it impacts NOI further.</t>
         </is>
       </c>
-      <c r="B7" s="63" t="n"/>
-      <c r="C7" s="63" t="n"/>
-      <c r="D7" s="63" t="n"/>
-      <c r="E7" s="63" t="n"/>
-      <c r="F7" s="63" t="n"/>
-      <c r="G7" s="63" t="n"/>
-      <c r="H7" s="63" t="n"/>
-      <c r="I7" s="63" t="n"/>
-      <c r="J7" s="63" t="n"/>
+      <c r="B7" s="64" t="n"/>
+      <c r="C7" s="64" t="n"/>
+      <c r="D7" s="64" t="n"/>
+      <c r="E7" s="64" t="n"/>
+      <c r="F7" s="64" t="n"/>
+      <c r="G7" s="64" t="n"/>
+      <c r="H7" s="64" t="n"/>
+      <c r="I7" s="64" t="n"/>
+      <c r="J7" s="64" t="n"/>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="62" t="inlineStr">
+      <c r="A9" s="63" t="inlineStr">
         <is>
           <t>MHC-03: Dual-Flag Asset Requiring Immediate Operational Review</t>
         </is>
       </c>
-      <c r="B9" s="63" t="n"/>
-      <c r="C9" s="63" t="n"/>
-      <c r="D9" s="63" t="n"/>
-      <c r="E9" s="63" t="n"/>
-      <c r="F9" s="63" t="n"/>
-      <c r="G9" s="63" t="n"/>
-      <c r="H9" s="63" t="n"/>
-      <c r="I9" s="63" t="n"/>
-      <c r="J9" s="63" t="n"/>
+      <c r="B9" s="64" t="n"/>
+      <c r="C9" s="64" t="n"/>
+      <c r="D9" s="64" t="n"/>
+      <c r="E9" s="64" t="n"/>
+      <c r="F9" s="64" t="n"/>
+      <c r="G9" s="64" t="n"/>
+      <c r="H9" s="64" t="n"/>
+      <c r="I9" s="64" t="n"/>
+      <c r="J9" s="64" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="64" t="inlineStr">
+      <c r="A10" s="65" t="inlineStr">
         <is>
           <t>Canyon Ridge | MHC | Low occupancy around 78–83% and high delinquency around 12–16%</t>
         </is>
       </c>
-      <c r="B10" s="63" t="n"/>
-      <c r="C10" s="63" t="n"/>
-      <c r="D10" s="63" t="n"/>
-      <c r="E10" s="63" t="n"/>
-      <c r="F10" s="63" t="n"/>
-      <c r="G10" s="63" t="n"/>
-      <c r="H10" s="63" t="n"/>
-      <c r="I10" s="63" t="n"/>
-      <c r="J10" s="63" t="n"/>
+      <c r="B10" s="64" t="n"/>
+      <c r="C10" s="64" t="n"/>
+      <c r="D10" s="64" t="n"/>
+      <c r="E10" s="64" t="n"/>
+      <c r="F10" s="64" t="n"/>
+      <c r="G10" s="64" t="n"/>
+      <c r="H10" s="64" t="n"/>
+      <c r="I10" s="64" t="n"/>
+      <c r="J10" s="64" t="n"/>
     </row>
     <row r="11" ht="55" customHeight="1">
-      <c r="A11" s="65" t="inlineStr">
+      <c r="A11" s="66" t="inlineStr">
         <is>
           <t>Data shows: MHC-03 is the weakest risk profile in the portfolio because it has both demand weakness and collections risk. This combination can pressure revenue, NOI, and investor reporting.</t>
         </is>
       </c>
-      <c r="B11" s="63" t="n"/>
-      <c r="C11" s="63" t="n"/>
-      <c r="D11" s="63" t="n"/>
-      <c r="E11" s="63" t="n"/>
-      <c r="F11" s="63" t="n"/>
-      <c r="G11" s="63" t="n"/>
-      <c r="H11" s="63" t="n"/>
-      <c r="I11" s="63" t="n"/>
-      <c r="J11" s="63" t="n"/>
+      <c r="B11" s="64" t="n"/>
+      <c r="C11" s="64" t="n"/>
+      <c r="D11" s="64" t="n"/>
+      <c r="E11" s="64" t="n"/>
+      <c r="F11" s="64" t="n"/>
+      <c r="G11" s="64" t="n"/>
+      <c r="H11" s="64" t="n"/>
+      <c r="I11" s="64" t="n"/>
+      <c r="J11" s="64" t="n"/>
     </row>
     <row r="12" ht="55" customHeight="1">
-      <c r="A12" s="66" t="inlineStr">
+      <c r="A12" s="67" t="inlineStr">
         <is>
           <t>Recommended action: Prioritize an operational review covering leasing activity, local market positioning, rent levels, resident retention, and collections. This property should be included in weekly asset management follow-up until both occupancy and delinquency stabilize.</t>
         </is>
       </c>
-      <c r="B12" s="63" t="n"/>
-      <c r="C12" s="63" t="n"/>
-      <c r="D12" s="63" t="n"/>
-      <c r="E12" s="63" t="n"/>
-      <c r="F12" s="63" t="n"/>
-      <c r="G12" s="63" t="n"/>
-      <c r="H12" s="63" t="n"/>
-      <c r="I12" s="63" t="n"/>
-      <c r="J12" s="63" t="n"/>
+      <c r="B12" s="64" t="n"/>
+      <c r="C12" s="64" t="n"/>
+      <c r="D12" s="64" t="n"/>
+      <c r="E12" s="64" t="n"/>
+      <c r="F12" s="64" t="n"/>
+      <c r="G12" s="64" t="n"/>
+      <c r="H12" s="64" t="n"/>
+      <c r="I12" s="64" t="n"/>
+      <c r="J12" s="64" t="n"/>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="62" t="inlineStr">
+      <c r="A14" s="63" t="inlineStr">
         <is>
           <t>MHC-04: Portfolio Benchmark — Operational Best Practices Template</t>
         </is>
       </c>
-      <c r="B14" s="63" t="n"/>
-      <c r="C14" s="63" t="n"/>
-      <c r="D14" s="63" t="n"/>
-      <c r="E14" s="63" t="n"/>
-      <c r="F14" s="63" t="n"/>
-      <c r="G14" s="63" t="n"/>
-      <c r="H14" s="63" t="n"/>
-      <c r="I14" s="63" t="n"/>
-      <c r="J14" s="63" t="n"/>
+      <c r="B14" s="64" t="n"/>
+      <c r="C14" s="64" t="n"/>
+      <c r="D14" s="64" t="n"/>
+      <c r="E14" s="64" t="n"/>
+      <c r="F14" s="64" t="n"/>
+      <c r="G14" s="64" t="n"/>
+      <c r="H14" s="64" t="n"/>
+      <c r="I14" s="64" t="n"/>
+      <c r="J14" s="64" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="64" t="inlineStr">
+      <c r="A15" s="65" t="inlineStr">
         <is>
           <t>Saguaro Estates | MHC | High occupancy, low delinquency, strong NOI margin</t>
         </is>
       </c>
-      <c r="B15" s="63" t="n"/>
-      <c r="C15" s="63" t="n"/>
-      <c r="D15" s="63" t="n"/>
-      <c r="E15" s="63" t="n"/>
-      <c r="F15" s="63" t="n"/>
-      <c r="G15" s="63" t="n"/>
-      <c r="H15" s="63" t="n"/>
-      <c r="I15" s="63" t="n"/>
-      <c r="J15" s="63" t="n"/>
+      <c r="B15" s="64" t="n"/>
+      <c r="C15" s="64" t="n"/>
+      <c r="D15" s="64" t="n"/>
+      <c r="E15" s="64" t="n"/>
+      <c r="F15" s="64" t="n"/>
+      <c r="G15" s="64" t="n"/>
+      <c r="H15" s="64" t="n"/>
+      <c r="I15" s="64" t="n"/>
+      <c r="J15" s="64" t="n"/>
     </row>
     <row r="16" ht="55" customHeight="1">
-      <c r="A16" s="65" t="inlineStr">
+      <c r="A16" s="66" t="inlineStr">
         <is>
           <t>Data shows: MHC-04 performs like a benchmark asset, with high occupancy, low delinquency, and strong profitability. This indicates strong property-level execution and stable resident demand.</t>
         </is>
       </c>
-      <c r="B16" s="63" t="n"/>
-      <c r="C16" s="63" t="n"/>
-      <c r="D16" s="63" t="n"/>
-      <c r="E16" s="63" t="n"/>
-      <c r="F16" s="63" t="n"/>
-      <c r="G16" s="63" t="n"/>
-      <c r="H16" s="63" t="n"/>
-      <c r="I16" s="63" t="n"/>
-      <c r="J16" s="63" t="n"/>
+      <c r="B16" s="64" t="n"/>
+      <c r="C16" s="64" t="n"/>
+      <c r="D16" s="64" t="n"/>
+      <c r="E16" s="64" t="n"/>
+      <c r="F16" s="64" t="n"/>
+      <c r="G16" s="64" t="n"/>
+      <c r="H16" s="64" t="n"/>
+      <c r="I16" s="64" t="n"/>
+      <c r="J16" s="64" t="n"/>
     </row>
     <row r="17" ht="55" customHeight="1">
-      <c r="A17" s="66" t="inlineStr">
+      <c r="A17" s="67" t="inlineStr">
         <is>
           <t>Recommended action: Use MHC-04 as an internal operating benchmark. Compare staffing, collections process, leasing practices, resident communication, and expense controls against weaker MHC assets.</t>
         </is>
       </c>
-      <c r="B17" s="63" t="n"/>
-      <c r="C17" s="63" t="n"/>
-      <c r="D17" s="63" t="n"/>
-      <c r="E17" s="63" t="n"/>
-      <c r="F17" s="63" t="n"/>
-      <c r="G17" s="63" t="n"/>
-      <c r="H17" s="63" t="n"/>
-      <c r="I17" s="63" t="n"/>
-      <c r="J17" s="63" t="n"/>
+      <c r="B17" s="64" t="n"/>
+      <c r="C17" s="64" t="n"/>
+      <c r="D17" s="64" t="n"/>
+      <c r="E17" s="64" t="n"/>
+      <c r="F17" s="64" t="n"/>
+      <c r="G17" s="64" t="n"/>
+      <c r="H17" s="64" t="n"/>
+      <c r="I17" s="64" t="n"/>
+      <c r="J17" s="64" t="n"/>
     </row>
     <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="62" t="inlineStr">
+      <c r="A19" s="63" t="inlineStr">
         <is>
           <t>MHC-05: Value-Add Play — Track Against Pro Forma Monthly</t>
         </is>
       </c>
-      <c r="B19" s="63" t="n"/>
-      <c r="C19" s="63" t="n"/>
-      <c r="D19" s="63" t="n"/>
-      <c r="E19" s="63" t="n"/>
-      <c r="F19" s="63" t="n"/>
-      <c r="G19" s="63" t="n"/>
-      <c r="H19" s="63" t="n"/>
-      <c r="I19" s="63" t="n"/>
-      <c r="J19" s="63" t="n"/>
+      <c r="B19" s="64" t="n"/>
+      <c r="C19" s="64" t="n"/>
+      <c r="D19" s="64" t="n"/>
+      <c r="E19" s="64" t="n"/>
+      <c r="F19" s="64" t="n"/>
+      <c r="G19" s="64" t="n"/>
+      <c r="H19" s="64" t="n"/>
+      <c r="I19" s="64" t="n"/>
+      <c r="J19" s="64" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="64" t="inlineStr">
+      <c r="A20" s="65" t="inlineStr">
         <is>
           <t>Pinon Pines | MHC | Occupancy improves from roughly 81% to 89% over the year</t>
         </is>
       </c>
-      <c r="B20" s="63" t="n"/>
-      <c r="C20" s="63" t="n"/>
-      <c r="D20" s="63" t="n"/>
-      <c r="E20" s="63" t="n"/>
-      <c r="F20" s="63" t="n"/>
-      <c r="G20" s="63" t="n"/>
-      <c r="H20" s="63" t="n"/>
-      <c r="I20" s="63" t="n"/>
-      <c r="J20" s="63" t="n"/>
+      <c r="B20" s="64" t="n"/>
+      <c r="C20" s="64" t="n"/>
+      <c r="D20" s="64" t="n"/>
+      <c r="E20" s="64" t="n"/>
+      <c r="F20" s="64" t="n"/>
+      <c r="G20" s="64" t="n"/>
+      <c r="H20" s="64" t="n"/>
+      <c r="I20" s="64" t="n"/>
+      <c r="J20" s="64" t="n"/>
     </row>
     <row r="21" ht="55" customHeight="1">
-      <c r="A21" s="65" t="inlineStr">
+      <c r="A21" s="66" t="inlineStr">
         <is>
           <t>Data shows: MHC-05 shows a positive value-add trend with improving occupancy, but it has not yet reached stabilized performance. The asset has rent upside and operational upside, making it a good candidate for active tracking.</t>
         </is>
       </c>
-      <c r="B21" s="63" t="n"/>
-      <c r="C21" s="63" t="n"/>
-      <c r="D21" s="63" t="n"/>
-      <c r="E21" s="63" t="n"/>
-      <c r="F21" s="63" t="n"/>
-      <c r="G21" s="63" t="n"/>
-      <c r="H21" s="63" t="n"/>
-      <c r="I21" s="63" t="n"/>
-      <c r="J21" s="63" t="n"/>
+      <c r="B21" s="64" t="n"/>
+      <c r="C21" s="64" t="n"/>
+      <c r="D21" s="64" t="n"/>
+      <c r="E21" s="64" t="n"/>
+      <c r="F21" s="64" t="n"/>
+      <c r="G21" s="64" t="n"/>
+      <c r="H21" s="64" t="n"/>
+      <c r="I21" s="64" t="n"/>
+      <c r="J21" s="64" t="n"/>
     </row>
     <row r="22" ht="55" customHeight="1">
-      <c r="A22" s="66" t="inlineStr">
+      <c r="A22" s="67" t="inlineStr">
         <is>
           <t>Recommended action: Track MHC-05 monthly against the acquisition pro forma, especially occupancy, rent growth, CapEx spend, and NOI margin. Management should confirm that renovation dollars are converting into occupancy gains and stronger cash flow.</t>
         </is>
       </c>
-      <c r="B22" s="63" t="n"/>
-      <c r="C22" s="63" t="n"/>
-      <c r="D22" s="63" t="n"/>
-      <c r="E22" s="63" t="n"/>
-      <c r="F22" s="63" t="n"/>
-      <c r="G22" s="63" t="n"/>
-      <c r="H22" s="63" t="n"/>
-      <c r="I22" s="63" t="n"/>
-      <c r="J22" s="63" t="n"/>
+      <c r="B22" s="64" t="n"/>
+      <c r="C22" s="64" t="n"/>
+      <c r="D22" s="64" t="n"/>
+      <c r="E22" s="64" t="n"/>
+      <c r="F22" s="64" t="n"/>
+      <c r="G22" s="64" t="n"/>
+      <c r="H22" s="64" t="n"/>
+      <c r="I22" s="64" t="n"/>
+      <c r="J22" s="64" t="n"/>
     </row>
     <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="62" t="inlineStr">
+      <c r="A24" s="63" t="inlineStr">
         <is>
           <t>STG-03: Expense Ratio Drag — NOI Underperformance Despite Adequate Occupancy</t>
         </is>
       </c>
-      <c r="B24" s="63" t="n"/>
-      <c r="C24" s="63" t="n"/>
-      <c r="D24" s="63" t="n"/>
-      <c r="E24" s="63" t="n"/>
-      <c r="F24" s="63" t="n"/>
-      <c r="G24" s="63" t="n"/>
-      <c r="H24" s="63" t="n"/>
-      <c r="I24" s="63" t="n"/>
-      <c r="J24" s="63" t="n"/>
+      <c r="B24" s="64" t="n"/>
+      <c r="C24" s="64" t="n"/>
+      <c r="D24" s="64" t="n"/>
+      <c r="E24" s="64" t="n"/>
+      <c r="F24" s="64" t="n"/>
+      <c r="G24" s="64" t="n"/>
+      <c r="H24" s="64" t="n"/>
+      <c r="I24" s="64" t="n"/>
+      <c r="J24" s="64" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="64" t="inlineStr">
+      <c r="A25" s="65" t="inlineStr">
         <is>
           <t>Desert Vault | Self-Storage | Expense ratio around 62–68%</t>
         </is>
       </c>
-      <c r="B25" s="63" t="n"/>
-      <c r="C25" s="63" t="n"/>
-      <c r="D25" s="63" t="n"/>
-      <c r="E25" s="63" t="n"/>
-      <c r="F25" s="63" t="n"/>
-      <c r="G25" s="63" t="n"/>
-      <c r="H25" s="63" t="n"/>
-      <c r="I25" s="63" t="n"/>
-      <c r="J25" s="63" t="n"/>
+      <c r="B25" s="64" t="n"/>
+      <c r="C25" s="64" t="n"/>
+      <c r="D25" s="64" t="n"/>
+      <c r="E25" s="64" t="n"/>
+      <c r="F25" s="64" t="n"/>
+      <c r="G25" s="64" t="n"/>
+      <c r="H25" s="64" t="n"/>
+      <c r="I25" s="64" t="n"/>
+      <c r="J25" s="64" t="n"/>
     </row>
     <row r="26" ht="55" customHeight="1">
-      <c r="A26" s="65" t="inlineStr">
+      <c r="A26" s="66" t="inlineStr">
         <is>
           <t>Data shows: STG-03 does not appear to be purely an occupancy problem. The high expense ratio is reducing NOI margin and making the property less profitable than it should be.</t>
         </is>
       </c>
-      <c r="B26" s="63" t="n"/>
-      <c r="C26" s="63" t="n"/>
-      <c r="D26" s="63" t="n"/>
-      <c r="E26" s="63" t="n"/>
-      <c r="F26" s="63" t="n"/>
-      <c r="G26" s="63" t="n"/>
-      <c r="H26" s="63" t="n"/>
-      <c r="I26" s="63" t="n"/>
-      <c r="J26" s="63" t="n"/>
+      <c r="B26" s="64" t="n"/>
+      <c r="C26" s="64" t="n"/>
+      <c r="D26" s="64" t="n"/>
+      <c r="E26" s="64" t="n"/>
+      <c r="F26" s="64" t="n"/>
+      <c r="G26" s="64" t="n"/>
+      <c r="H26" s="64" t="n"/>
+      <c r="I26" s="64" t="n"/>
+      <c r="J26" s="64" t="n"/>
     </row>
     <row r="27" ht="55" customHeight="1">
-      <c r="A27" s="66" t="inlineStr">
+      <c r="A27" s="67" t="inlineStr">
         <is>
           <t>Recommended action: Review controllable expenses such as repairs, payroll, utilities, vendor contracts, insurance, and recurring maintenance. The finance and asset management teams should isolate which expense categories are driving margin compression.</t>
         </is>
       </c>
-      <c r="B27" s="63" t="n"/>
-      <c r="C27" s="63" t="n"/>
-      <c r="D27" s="63" t="n"/>
-      <c r="E27" s="63" t="n"/>
-      <c r="F27" s="63" t="n"/>
-      <c r="G27" s="63" t="n"/>
-      <c r="H27" s="63" t="n"/>
-      <c r="I27" s="63" t="n"/>
-      <c r="J27" s="63" t="n"/>
+      <c r="B27" s="64" t="n"/>
+      <c r="C27" s="64" t="n"/>
+      <c r="D27" s="64" t="n"/>
+      <c r="E27" s="64" t="n"/>
+      <c r="F27" s="64" t="n"/>
+      <c r="G27" s="64" t="n"/>
+      <c r="H27" s="64" t="n"/>
+      <c r="I27" s="64" t="n"/>
+      <c r="J27" s="64" t="n"/>
     </row>
     <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="62" t="inlineStr">
+      <c r="A29" s="63" t="inlineStr">
         <is>
           <t>MHC-07: Early Warning — Delinquency Trend Requires Collections Intervention Before It Escalates</t>
         </is>
       </c>
-      <c r="B29" s="63" t="n"/>
-      <c r="C29" s="63" t="n"/>
-      <c r="D29" s="63" t="n"/>
-      <c r="E29" s="63" t="n"/>
-      <c r="F29" s="63" t="n"/>
-      <c r="G29" s="63" t="n"/>
-      <c r="H29" s="63" t="n"/>
-      <c r="I29" s="63" t="n"/>
-      <c r="J29" s="63" t="n"/>
+      <c r="B29" s="64" t="n"/>
+      <c r="C29" s="64" t="n"/>
+      <c r="D29" s="64" t="n"/>
+      <c r="E29" s="64" t="n"/>
+      <c r="F29" s="64" t="n"/>
+      <c r="G29" s="64" t="n"/>
+      <c r="H29" s="64" t="n"/>
+      <c r="I29" s="64" t="n"/>
+      <c r="J29" s="64" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="64" t="inlineStr">
+      <c r="A30" s="65" t="inlineStr">
         <is>
           <t>Mesa Vista | MHC | High occupancy but delinquency rising from approximately 5% to 11%</t>
         </is>
       </c>
-      <c r="B30" s="63" t="n"/>
-      <c r="C30" s="63" t="n"/>
-      <c r="D30" s="63" t="n"/>
-      <c r="E30" s="63" t="n"/>
-      <c r="F30" s="63" t="n"/>
-      <c r="G30" s="63" t="n"/>
-      <c r="H30" s="63" t="n"/>
-      <c r="I30" s="63" t="n"/>
-      <c r="J30" s="63" t="n"/>
+      <c r="B30" s="64" t="n"/>
+      <c r="C30" s="64" t="n"/>
+      <c r="D30" s="64" t="n"/>
+      <c r="E30" s="64" t="n"/>
+      <c r="F30" s="64" t="n"/>
+      <c r="G30" s="64" t="n"/>
+      <c r="H30" s="64" t="n"/>
+      <c r="I30" s="64" t="n"/>
+      <c r="J30" s="64" t="n"/>
     </row>
     <row r="31" ht="55" customHeight="1">
-      <c r="A31" s="65" t="inlineStr">
+      <c r="A31" s="66" t="inlineStr">
         <is>
           <t>Data shows: MHC-07 still has strong occupancy, but the delinquency trend is moving in the wrong direction. This is an early warning sign because the property looks healthy from an occupancy view but has growing collection risk.</t>
         </is>
       </c>
-      <c r="B31" s="63" t="n"/>
-      <c r="C31" s="63" t="n"/>
-      <c r="D31" s="63" t="n"/>
-      <c r="E31" s="63" t="n"/>
-      <c r="F31" s="63" t="n"/>
-      <c r="G31" s="63" t="n"/>
-      <c r="H31" s="63" t="n"/>
-      <c r="I31" s="63" t="n"/>
-      <c r="J31" s="63" t="n"/>
+      <c r="B31" s="64" t="n"/>
+      <c r="C31" s="64" t="n"/>
+      <c r="D31" s="64" t="n"/>
+      <c r="E31" s="64" t="n"/>
+      <c r="F31" s="64" t="n"/>
+      <c r="G31" s="64" t="n"/>
+      <c r="H31" s="64" t="n"/>
+      <c r="I31" s="64" t="n"/>
+      <c r="J31" s="64" t="n"/>
     </row>
     <row r="32" ht="55" customHeight="1">
-      <c r="A32" s="66" t="inlineStr">
+      <c r="A32" s="67" t="inlineStr">
         <is>
           <t>Recommended action: Intervene before the issue becomes critical by reviewing tenant aging buckets, payment plan usage, late-fee timing, and property manager follow-up. This should be treated as a collections process issue before assuming a demand issue.</t>
         </is>
       </c>
-      <c r="B32" s="63" t="n"/>
-      <c r="C32" s="63" t="n"/>
-      <c r="D32" s="63" t="n"/>
-      <c r="E32" s="63" t="n"/>
-      <c r="F32" s="63" t="n"/>
-      <c r="G32" s="63" t="n"/>
-      <c r="H32" s="63" t="n"/>
-      <c r="I32" s="63" t="n"/>
-      <c r="J32" s="63" t="n"/>
+      <c r="B32" s="64" t="n"/>
+      <c r="C32" s="64" t="n"/>
+      <c r="D32" s="64" t="n"/>
+      <c r="E32" s="64" t="n"/>
+      <c r="F32" s="64" t="n"/>
+      <c r="G32" s="64" t="n"/>
+      <c r="H32" s="64" t="n"/>
+      <c r="I32" s="64" t="n"/>
+      <c r="J32" s="64" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -18919,15 +18940,15 @@
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
     <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -18998,28 +19019,34 @@
       <c r="L4" s="27" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="n">
-        <v>12</v>
+      <c r="A5" s="30">
+        <f>COUNTA(Properties!A2:A1000)</f>
+        <v/>
       </c>
       <c r="B5" s="27" t="n"/>
-      <c r="C5" s="36" t="n">
-        <v>2065</v>
+      <c r="C5" s="36">
+        <f>SUM(Properties!F:F)</f>
+        <v/>
       </c>
       <c r="D5" s="27" t="n"/>
-      <c r="E5" s="37" t="n">
-        <v>0.910411622276029</v>
+      <c r="E5" s="37">
+        <f>SUMIFS(Occupancy!E:E,Occupancy!D:D,MAX(Occupancy!D:D))/SUMIFS(Occupancy!F:F,Occupancy!D:D,MAX(Occupancy!D:D))</f>
+        <v/>
       </c>
       <c r="F5" s="27" t="n"/>
-      <c r="G5" s="28" t="n">
-        <v>329033.8900000001</v>
+      <c r="G5" s="28">
+        <f>SUMIFS(Financials!G:G,Financials!D:D,MAX(Financials!D:D))</f>
+        <v/>
       </c>
       <c r="H5" s="27" t="n"/>
-      <c r="I5" s="37" t="n">
-        <v>0.07867780106626204</v>
+      <c r="I5" s="37">
+        <f>SUMIFS(Delinquency!G:G,Delinquency!D:D,MAX(Delinquency!D:D))/SUMIFS(Delinquency!E:E,Delinquency!D:D,MAX(Delinquency!D:D))</f>
+        <v/>
       </c>
       <c r="J5" s="27" t="n"/>
-      <c r="K5" s="28" t="n">
-        <v>111500000</v>
+      <c r="K5" s="28">
+        <f>SUM(Properties!H:H)</f>
+        <v/>
       </c>
       <c r="L5" s="27" t="n"/>
     </row>
@@ -19065,9 +19092,15 @@
       <c r="K8" s="27" t="n"/>
       <c r="L8" s="27" t="n"/>
     </row>
-    <row r="9"/>
+    <row r="9">
+      <c r="A9" s="38" t="inlineStr">
+        <is>
+          <t>Dashboard metrics are formula-driven from source tabs where practical.</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
-      <c r="A10" s="38" t="inlineStr">
+      <c r="A10" s="39" t="inlineStr">
         <is>
           <t>Asset Type Comparison</t>
         </is>
@@ -19159,7 +19192,7 @@
     <row r="18"/>
     <row r="19"/>
     <row r="20">
-      <c r="A20" s="38" t="inlineStr">
+      <c r="A20" s="39" t="inlineStr">
         <is>
           <t>Properties Requiring Attention — Most Recent Month</t>
         </is>
@@ -19225,7 +19258,7 @@
       <c r="F22" s="15" t="n">
         <v>0.4895</v>
       </c>
-      <c r="G22" s="39" t="inlineStr">
+      <c r="G22" s="40" t="inlineStr">
         <is>
           <t>HIGH RISK</t>
         </is>
@@ -19254,7 +19287,7 @@
       <c r="F23" s="15" t="n">
         <v>0.4216</v>
       </c>
-      <c r="G23" s="40" t="inlineStr">
+      <c r="G23" s="41" t="inlineStr">
         <is>
           <t>DELINQUENCY RISK</t>
         </is>
@@ -19283,7 +19316,7 @@
       <c r="F24" s="15" t="n">
         <v>0.5009</v>
       </c>
-      <c r="G24" s="40" t="inlineStr">
+      <c r="G24" s="41" t="inlineStr">
         <is>
           <t>DELINQUENCY RISK</t>
         </is>
@@ -19312,7 +19345,7 @@
       <c r="F25" s="15" t="n">
         <v>0.5069</v>
       </c>
-      <c r="G25" s="41" t="inlineStr">
+      <c r="G25" s="42" t="inlineStr">
         <is>
           <t>OCCUPANCY RISK</t>
         </is>
@@ -19341,7 +19374,7 @@
       <c r="F26" s="15" t="n">
         <v>0.4719</v>
       </c>
-      <c r="G26" s="41" t="inlineStr">
+      <c r="G26" s="42" t="inlineStr">
         <is>
           <t>OCCUPANCY RISK</t>
         </is>
@@ -19370,7 +19403,7 @@
       <c r="F27" s="15" t="n">
         <v>0.386</v>
       </c>
-      <c r="G27" s="41" t="inlineStr">
+      <c r="G27" s="42" t="inlineStr">
         <is>
           <t>OCCUPANCY RISK</t>
         </is>
@@ -19378,7 +19411,7 @@
     </row>
     <row r="28"/>
     <row r="29">
-      <c r="A29" s="42" t="inlineStr">
+      <c r="A29" s="43" t="inlineStr">
         <is>
           <t>This exception report combines occupancy, collections risk, and NOI to help asset managers prioritize follow-up.</t>
         </is>
@@ -19386,12 +19419,12 @@
     </row>
     <row r="30"/>
     <row r="31">
-      <c r="A31" s="43" t="inlineStr">
+      <c r="A31" s="44" t="inlineStr">
         <is>
           <t>Top 5 Properties by NOI Margin</t>
         </is>
       </c>
-      <c r="F31" s="43" t="inlineStr">
+      <c r="F31" s="44" t="inlineStr">
         <is>
           <t>Bottom 5 Properties by NOI Margin</t>
         </is>
@@ -19430,17 +19463,17 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="44" t="inlineStr">
+      <c r="A33" s="45" t="inlineStr">
         <is>
           <t>Saguaro Estates</t>
         </is>
       </c>
-      <c r="B33" s="44" t="inlineStr">
-        <is>
-          <t>MHC</t>
-        </is>
-      </c>
-      <c r="C33" s="45" t="n">
+      <c r="B33" s="45" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C33" s="46" t="n">
         <v>0.5849</v>
       </c>
       <c r="D33" s="13" t="n"/>
@@ -19460,17 +19493,17 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="44" t="inlineStr">
+      <c r="A34" s="45" t="inlineStr">
         <is>
           <t>Red Rock Commons</t>
         </is>
       </c>
-      <c r="B34" s="44" t="inlineStr">
-        <is>
-          <t>MHC</t>
-        </is>
-      </c>
-      <c r="C34" s="45" t="n">
+      <c r="B34" s="45" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C34" s="46" t="n">
         <v>0.536</v>
       </c>
       <c r="D34" s="13" t="n"/>
@@ -19490,17 +19523,17 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="44" t="inlineStr">
+      <c r="A35" s="45" t="inlineStr">
         <is>
           <t>Sunrise Meadows</t>
         </is>
       </c>
-      <c r="B35" s="44" t="inlineStr">
-        <is>
-          <t>MHC</t>
-        </is>
-      </c>
-      <c r="C35" s="45" t="n">
+      <c r="B35" s="45" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C35" s="46" t="n">
         <v>0.5152</v>
       </c>
       <c r="D35" s="13" t="n"/>
@@ -19520,17 +19553,17 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="44" t="inlineStr">
+      <c r="A36" s="45" t="inlineStr">
         <is>
           <t>Desert Palms</t>
         </is>
       </c>
-      <c r="B36" s="44" t="inlineStr">
-        <is>
-          <t>MHC</t>
-        </is>
-      </c>
-      <c r="C36" s="45" t="n">
+      <c r="B36" s="45" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C36" s="46" t="n">
         <v>0.5069</v>
       </c>
       <c r="D36" s="13" t="n"/>
@@ -19550,17 +19583,17 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="44" t="inlineStr">
+      <c r="A37" s="45" t="inlineStr">
         <is>
           <t>Mesa Vista</t>
         </is>
       </c>
-      <c r="B37" s="44" t="inlineStr">
-        <is>
-          <t>MHC</t>
-        </is>
-      </c>
-      <c r="C37" s="45" t="n">
+      <c r="B37" s="45" t="inlineStr">
+        <is>
+          <t>MHC</t>
+        </is>
+      </c>
+      <c r="C37" s="46" t="n">
         <v>0.5009</v>
       </c>
       <c r="D37" s="13" t="n"/>
@@ -19580,7 +19613,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
     <mergeCell ref="I3:J4"/>
     <mergeCell ref="A20:G20"/>
     <mergeCell ref="G5:H8"/>
@@ -19595,6 +19628,7 @@
     <mergeCell ref="A29:I29"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="C5:D8"/>
+    <mergeCell ref="A9:L9"/>
     <mergeCell ref="K5:L8"/>
     <mergeCell ref="E5:F8"/>
     <mergeCell ref="A1:L1"/>
@@ -19612,33 +19646,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="46" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>Acquisition Underwriting — MHC-05 Pinon Pines</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="47" t="inlineStr">
+      <c r="A2" s="48" t="inlineStr">
         <is>
           <t>Underwriting Assumptions</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="48" t="inlineStr">
+      <c r="A3" s="49" t="inlineStr">
         <is>
           <t>Assumption</t>
         </is>
@@ -19652,158 +19687,179 @@
     <row r="4">
       <c r="A4" s="50" t="inlineStr">
         <is>
-          <t>Total Units</t>
+          <t>Purchase Price</t>
         </is>
       </c>
       <c r="B4" s="51" t="n">
-        <v>88</v>
+        <v>4200000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="50" t="inlineStr">
         <is>
-          <t>Current Occupancy</t>
+          <t>Total Units</t>
         </is>
       </c>
       <c r="B5" s="52" t="n">
-        <v>0.82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="50" t="inlineStr">
         <is>
-          <t>Stabilized Occupancy Target</t>
-        </is>
-      </c>
-      <c r="B6" s="52" t="n">
-        <v>0.93</v>
+          <t>Current Occupancy</t>
+        </is>
+      </c>
+      <c r="B6" s="53" t="n">
+        <v>0.82</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="50" t="inlineStr">
         <is>
-          <t>Current Avg Monthly Rent per Lot</t>
+          <t>Stabilized Occupancy Target</t>
         </is>
       </c>
       <c r="B7" s="53" t="n">
-        <v>720</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="50" t="inlineStr">
         <is>
-          <t>Market Avg Rent</t>
-        </is>
-      </c>
-      <c r="B8" s="53" t="n">
-        <v>810</v>
+          <t>Current Avg Monthly Rent per Lot</t>
+        </is>
+      </c>
+      <c r="B8" s="51" t="n">
+        <v>720</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="50" t="inlineStr">
         <is>
-          <t>Year 1 Rent Growth</t>
-        </is>
-      </c>
-      <c r="B9" s="52" t="n">
-        <v>0.045</v>
+          <t>Market Avg Rent</t>
+        </is>
+      </c>
+      <c r="B9" s="51" t="n">
+        <v>810</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="50" t="inlineStr">
         <is>
-          <t>Years 2-5 Rent Growth</t>
-        </is>
-      </c>
-      <c r="B10" s="52" t="n">
-        <v>0.03</v>
+          <t>Year 1 Rent Growth</t>
+        </is>
+      </c>
+      <c r="B10" s="53" t="n">
+        <v>0.045</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="50" t="inlineStr">
         <is>
-          <t>Operating Expense Ratio Year 1</t>
-        </is>
-      </c>
-      <c r="B11" s="52" t="n">
-        <v>0.48</v>
+          <t>Years 2-5 Rent Growth</t>
+        </is>
+      </c>
+      <c r="B11" s="53" t="n">
+        <v>0.03</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="50" t="inlineStr">
         <is>
-          <t>Expense Ratio Improvement</t>
-        </is>
-      </c>
-      <c r="B12" s="52" t="n">
-        <v>-0.01</v>
+          <t>Operating Expense Ratio Year 1</t>
+        </is>
+      </c>
+      <c r="B12" s="53" t="n">
+        <v>0.48</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="50" t="inlineStr">
         <is>
-          <t>Renovation CapEx Year 1</t>
+          <t>Expense Ratio Improvement</t>
         </is>
       </c>
       <c r="B13" s="53" t="n">
-        <v>380000</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="50" t="inlineStr">
         <is>
-          <t>Exit Cap Rate</t>
-        </is>
-      </c>
-      <c r="B14" s="54" t="n">
-        <v>0.0625</v>
+          <t>Renovation CapEx Year 1</t>
+        </is>
+      </c>
+      <c r="B14" s="51" t="n">
+        <v>380000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="50" t="inlineStr">
         <is>
-          <t>Loan Amount</t>
-        </is>
-      </c>
-      <c r="B15" s="53" t="n">
-        <v>2730000</v>
+          <t>Exit Cap Rate</t>
+        </is>
+      </c>
+      <c r="B15" s="54" t="n">
+        <v>0.0625</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="50" t="inlineStr">
         <is>
-          <t>Interest Rate</t>
-        </is>
-      </c>
-      <c r="B16" s="52" t="n">
-        <v>0.068</v>
+          <t>Loan Amount</t>
+        </is>
+      </c>
+      <c r="B16" s="51">
+        <f>B4*65%</f>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="50" t="inlineStr">
         <is>
-          <t>Loan Term</t>
-        </is>
-      </c>
-      <c r="B17" s="51" t="n">
-        <v>10</v>
+          <t>Interest Rate</t>
+        </is>
+      </c>
+      <c r="B17" s="53" t="n">
+        <v>0.068</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="50" t="inlineStr">
         <is>
+          <t>Loan Term</t>
+        </is>
+      </c>
+      <c r="B18" s="52" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="50" t="inlineStr">
+        <is>
           <t>Acquisition Costs</t>
         </is>
       </c>
-      <c r="B18" s="52" t="n">
-        <v>0.025</v>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20"/>
+      <c r="B19" s="51">
+        <f>B4*2.5%</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="50" t="inlineStr">
+        <is>
+          <t>Initial Equity</t>
+        </is>
+      </c>
+      <c r="B20" s="51">
+        <f>B4-B16+B14+B19</f>
+        <v/>
+      </c>
+    </row>
     <row r="21"/>
     <row r="22">
-      <c r="A22" s="47" t="inlineStr">
+      <c r="A22" s="48" t="inlineStr">
         <is>
           <t>5-Year Operating Pro Forma</t>
         </is>
@@ -19847,20 +19903,25 @@
           <t>Occupied Units</t>
         </is>
       </c>
-      <c r="B24" s="55" t="n">
-        <v>74</v>
-      </c>
-      <c r="C24" s="55" t="n">
-        <v>76</v>
-      </c>
-      <c r="D24" s="55" t="n">
-        <v>78</v>
-      </c>
-      <c r="E24" s="55" t="n">
-        <v>80</v>
-      </c>
-      <c r="F24" s="55" t="n">
-        <v>82</v>
+      <c r="B24" s="55">
+        <f>$B$5*B25</f>
+        <v/>
+      </c>
+      <c r="C24" s="55">
+        <f>$B$5*C25</f>
+        <v/>
+      </c>
+      <c r="D24" s="55">
+        <f>$B$5*D25</f>
+        <v/>
+      </c>
+      <c r="E24" s="55">
+        <f>$B$5*E25</f>
+        <v/>
+      </c>
+      <c r="F24" s="55">
+        <f>$B$5*F25</f>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -19869,20 +19930,25 @@
           <t>Occupancy Rate</t>
         </is>
       </c>
-      <c r="B25" s="56" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="C25" s="56" t="n">
-        <v>0.865</v>
-      </c>
-      <c r="D25" s="56" t="n">
-        <v>0.89</v>
-      </c>
-      <c r="E25" s="56" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="F25" s="56" t="n">
-        <v>0.93</v>
+      <c r="B25" s="56">
+        <f>MAX(84%,$B$6+2%)</f>
+        <v/>
+      </c>
+      <c r="C25" s="56">
+        <f>B25+($B$7-B25)/4</f>
+        <v/>
+      </c>
+      <c r="D25" s="56">
+        <f>C25+($B$7-B25)/4</f>
+        <v/>
+      </c>
+      <c r="E25" s="56">
+        <f>D25+($B$7-B25)/4</f>
+        <v/>
+      </c>
+      <c r="F25" s="56">
+        <f>$B$7</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -19891,20 +19957,25 @@
           <t>Avg Monthly Rent</t>
         </is>
       </c>
-      <c r="B26" s="57" t="n">
-        <v>752.4</v>
-      </c>
-      <c r="C26" s="57" t="n">
-        <v>774.972</v>
-      </c>
-      <c r="D26" s="57" t="n">
-        <v>798.2211600000001</v>
-      </c>
-      <c r="E26" s="57" t="n">
-        <v>822.1677948</v>
-      </c>
-      <c r="F26" s="57" t="n">
-        <v>846.8328286440001</v>
+      <c r="B26" s="57">
+        <f>$B$8*(1+$B$10)</f>
+        <v/>
+      </c>
+      <c r="C26" s="57">
+        <f>B26*(1+$B$11)</f>
+        <v/>
+      </c>
+      <c r="D26" s="57">
+        <f>C26*(1+$B$11)</f>
+        <v/>
+      </c>
+      <c r="E26" s="57">
+        <f>D26*(1+$B$11)</f>
+        <v/>
+      </c>
+      <c r="F26" s="57">
+        <f>E26*(1+$B$11)</f>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -19913,20 +19984,25 @@
           <t>Gross Potential Rent Annual</t>
         </is>
       </c>
-      <c r="B27" s="57" t="n">
-        <v>794534.3999999999</v>
-      </c>
-      <c r="C27" s="57" t="n">
-        <v>818370.4319999999</v>
-      </c>
-      <c r="D27" s="57" t="n">
-        <v>842921.54496</v>
-      </c>
-      <c r="E27" s="57" t="n">
-        <v>868209.1913088</v>
-      </c>
-      <c r="F27" s="57" t="n">
-        <v>894255.467048064</v>
+      <c r="B27" s="57">
+        <f>$B$5*B26*12</f>
+        <v/>
+      </c>
+      <c r="C27" s="57">
+        <f>$B$5*C26*12</f>
+        <v/>
+      </c>
+      <c r="D27" s="57">
+        <f>$B$5*D26*12</f>
+        <v/>
+      </c>
+      <c r="E27" s="57">
+        <f>$B$5*E26*12</f>
+        <v/>
+      </c>
+      <c r="F27" s="57">
+        <f>$B$5*F26*12</f>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -19935,20 +20011,25 @@
           <t>Vacancy Loss</t>
         </is>
       </c>
-      <c r="B28" s="57" t="n">
-        <v>127125.504</v>
-      </c>
-      <c r="C28" s="57" t="n">
-        <v>110480.00832</v>
-      </c>
-      <c r="D28" s="57" t="n">
-        <v>92721.36994559999</v>
-      </c>
-      <c r="E28" s="57" t="n">
-        <v>78138.82721779197</v>
-      </c>
-      <c r="F28" s="57" t="n">
-        <v>62597.88269336444</v>
+      <c r="B28" s="57">
+        <f>B27*(1-B25)</f>
+        <v/>
+      </c>
+      <c r="C28" s="57">
+        <f>C27*(1-C25)</f>
+        <v/>
+      </c>
+      <c r="D28" s="57">
+        <f>D27*(1-D25)</f>
+        <v/>
+      </c>
+      <c r="E28" s="57">
+        <f>E27*(1-E25)</f>
+        <v/>
+      </c>
+      <c r="F28" s="57">
+        <f>F27*(1-F25)</f>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -19957,20 +20038,25 @@
           <t>Effective Gross Income</t>
         </is>
       </c>
-      <c r="B29" s="57" t="n">
-        <v>667408.8959999999</v>
-      </c>
-      <c r="C29" s="57" t="n">
-        <v>707890.4236799999</v>
-      </c>
-      <c r="D29" s="57" t="n">
-        <v>750200.1750143999</v>
-      </c>
-      <c r="E29" s="57" t="n">
-        <v>790070.3640910081</v>
-      </c>
-      <c r="F29" s="57" t="n">
-        <v>831657.5843546996</v>
+      <c r="B29" s="57">
+        <f>B27-B28</f>
+        <v/>
+      </c>
+      <c r="C29" s="57">
+        <f>C27-C28</f>
+        <v/>
+      </c>
+      <c r="D29" s="57">
+        <f>D27-D28</f>
+        <v/>
+      </c>
+      <c r="E29" s="57">
+        <f>E27-E28</f>
+        <v/>
+      </c>
+      <c r="F29" s="57">
+        <f>F27-F28</f>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -19979,20 +20065,25 @@
           <t>Operating Expenses</t>
         </is>
       </c>
-      <c r="B30" s="57" t="n">
-        <v>320356.27008</v>
-      </c>
-      <c r="C30" s="57" t="n">
-        <v>332708.4991295999</v>
-      </c>
-      <c r="D30" s="57" t="n">
-        <v>345092.080506624</v>
-      </c>
-      <c r="E30" s="57" t="n">
-        <v>355531.6638409536</v>
-      </c>
-      <c r="F30" s="57" t="n">
-        <v>365929.3371160678</v>
+      <c r="B30" s="57">
+        <f>B29*($B$12+(COLUMN(B30)-COLUMN($B$30))*$B$13)</f>
+        <v/>
+      </c>
+      <c r="C30" s="57">
+        <f>C29*($B$12+(COLUMN(C30)-COLUMN($B$30))*$B$13)</f>
+        <v/>
+      </c>
+      <c r="D30" s="57">
+        <f>D29*($B$12+(COLUMN(D30)-COLUMN($B$30))*$B$13)</f>
+        <v/>
+      </c>
+      <c r="E30" s="57">
+        <f>E29*($B$12+(COLUMN(E30)-COLUMN($B$30))*$B$13)</f>
+        <v/>
+      </c>
+      <c r="F30" s="57">
+        <f>F29*($B$12+(COLUMN(F30)-COLUMN($B$30))*$B$13)</f>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -20001,20 +20092,25 @@
           <t>NOI</t>
         </is>
       </c>
-      <c r="B31" s="57" t="n">
-        <v>347052.62592</v>
-      </c>
-      <c r="C31" s="57" t="n">
-        <v>375181.9245503999</v>
-      </c>
-      <c r="D31" s="57" t="n">
-        <v>405108.094507776</v>
-      </c>
-      <c r="E31" s="57" t="n">
-        <v>434538.7002500545</v>
-      </c>
-      <c r="F31" s="57" t="n">
-        <v>465728.2472386318</v>
+      <c r="B31" s="57">
+        <f>B29-B30</f>
+        <v/>
+      </c>
+      <c r="C31" s="57">
+        <f>C29-C30</f>
+        <v/>
+      </c>
+      <c r="D31" s="57">
+        <f>D29-D30</f>
+        <v/>
+      </c>
+      <c r="E31" s="57">
+        <f>E29-E30</f>
+        <v/>
+      </c>
+      <c r="F31" s="57">
+        <f>F29-F30</f>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -20023,20 +20119,25 @@
           <t>NOI Margin %</t>
         </is>
       </c>
-      <c r="B32" s="56" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="C32" s="56" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="D32" s="56" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="E32" s="56" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F32" s="56" t="n">
-        <v>0.5599999999999999</v>
+      <c r="B32" s="56">
+        <f>IFERROR(B31/B29,0)</f>
+        <v/>
+      </c>
+      <c r="C32" s="56">
+        <f>IFERROR(C31/C29,0)</f>
+        <v/>
+      </c>
+      <c r="D32" s="56">
+        <f>IFERROR(D31/D29,0)</f>
+        <v/>
+      </c>
+      <c r="E32" s="56">
+        <f>IFERROR(E31/E29,0)</f>
+        <v/>
+      </c>
+      <c r="F32" s="56">
+        <f>IFERROR(F31/F29,0)</f>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -20045,20 +20146,25 @@
           <t>Debt Service Annual P&amp;I</t>
         </is>
       </c>
-      <c r="B33" s="57" t="n">
-        <v>385104.9324103267</v>
-      </c>
-      <c r="C33" s="57" t="n">
-        <v>385104.9324103267</v>
-      </c>
-      <c r="D33" s="57" t="n">
-        <v>385104.9324103267</v>
-      </c>
-      <c r="E33" s="57" t="n">
-        <v>385104.9324103267</v>
-      </c>
-      <c r="F33" s="57" t="n">
-        <v>385104.9324103267</v>
+      <c r="B33" s="57">
+        <f>-PMT($B$17,$B$18,$B$16)</f>
+        <v/>
+      </c>
+      <c r="C33" s="57">
+        <f>-PMT($B$17,$B$18,$B$16)</f>
+        <v/>
+      </c>
+      <c r="D33" s="57">
+        <f>-PMT($B$17,$B$18,$B$16)</f>
+        <v/>
+      </c>
+      <c r="E33" s="57">
+        <f>-PMT($B$17,$B$18,$B$16)</f>
+        <v/>
+      </c>
+      <c r="F33" s="57">
+        <f>-PMT($B$17,$B$18,$B$16)</f>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -20067,20 +20173,25 @@
           <t>Net Cash Flow After Debt</t>
         </is>
       </c>
-      <c r="B34" s="57" t="n">
-        <v>-38052.30649032677</v>
-      </c>
-      <c r="C34" s="57" t="n">
-        <v>-9923.007859926787</v>
-      </c>
-      <c r="D34" s="57" t="n">
-        <v>20003.16209744924</v>
-      </c>
-      <c r="E34" s="57" t="n">
-        <v>49433.76783972775</v>
-      </c>
-      <c r="F34" s="57" t="n">
-        <v>80623.31482830504</v>
+      <c r="B34" s="57">
+        <f>B31-B33</f>
+        <v/>
+      </c>
+      <c r="C34" s="57">
+        <f>C31-C33</f>
+        <v/>
+      </c>
+      <c r="D34" s="57">
+        <f>D31-D33</f>
+        <v/>
+      </c>
+      <c r="E34" s="57">
+        <f>E31-E33</f>
+        <v/>
+      </c>
+      <c r="F34" s="57">
+        <f>F31-F33</f>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -20089,20 +20200,25 @@
           <t>Cash-on-Cash Return</t>
         </is>
       </c>
-      <c r="B35" s="56" t="n">
-        <v>-0.01946409539147149</v>
-      </c>
-      <c r="C35" s="56" t="n">
-        <v>-0.005075707345231093</v>
-      </c>
-      <c r="D35" s="56" t="n">
-        <v>0.0102317964692835</v>
-      </c>
-      <c r="E35" s="56" t="n">
-        <v>0.0252858147517789</v>
-      </c>
-      <c r="F35" s="56" t="n">
-        <v>0.0412395472267545</v>
+      <c r="B35" s="56">
+        <f>IFERROR(B34/$B$20,0)</f>
+        <v/>
+      </c>
+      <c r="C35" s="56">
+        <f>IFERROR(C34/$B$20,0)</f>
+        <v/>
+      </c>
+      <c r="D35" s="56">
+        <f>IFERROR(D34/$B$20,0)</f>
+        <v/>
+      </c>
+      <c r="E35" s="56">
+        <f>IFERROR(E34/$B$20,0)</f>
+        <v/>
+      </c>
+      <c r="F35" s="56">
+        <f>IFERROR(F34/$B$20,0)</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -20111,20 +20227,25 @@
           <t>Cumulative Cash Flow</t>
         </is>
       </c>
-      <c r="B36" s="57" t="n">
-        <v>-38052.30649032677</v>
-      </c>
-      <c r="C36" s="57" t="n">
-        <v>-47975.31435025355</v>
-      </c>
-      <c r="D36" s="57" t="n">
-        <v>-27972.15225280431</v>
-      </c>
-      <c r="E36" s="57" t="n">
-        <v>21461.61558692344</v>
-      </c>
-      <c r="F36" s="57" t="n">
-        <v>102084.9304152285</v>
+      <c r="B36" s="57">
+        <f>B34</f>
+        <v/>
+      </c>
+      <c r="C36" s="57">
+        <f>B36+C34</f>
+        <v/>
+      </c>
+      <c r="D36" s="57">
+        <f>C36+D34</f>
+        <v/>
+      </c>
+      <c r="E36" s="57">
+        <f>D36+E34</f>
+        <v/>
+      </c>
+      <c r="F36" s="57">
+        <f>E36+F34</f>
+        <v/>
       </c>
     </row>
     <row r="37"/>
@@ -20142,8 +20263,9 @@
           <t>Year 5 Exit Value</t>
         </is>
       </c>
-      <c r="B40" s="57" t="n">
-        <v>7451651.955818108</v>
+      <c r="B40" s="57">
+        <f>F31/$B$15</f>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -20152,8 +20274,9 @@
           <t>Remaining Loan Balance after 5 years</t>
         </is>
       </c>
-      <c r="B41" s="57" t="n">
-        <v>1587498.069811833</v>
+      <c r="B41" s="57">
+        <f>$B$16*(1+$B$17)^5-B33*(((1+$B$17)^5-1)/$B$17)</f>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -20162,8 +20285,9 @@
           <t>Net Proceeds</t>
         </is>
       </c>
-      <c r="B42" s="57" t="n">
-        <v>5864153.886006275</v>
+      <c r="B42" s="57">
+        <f>B41-B42</f>
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -20172,8 +20296,9 @@
           <t>Cumulative Cash Flow</t>
         </is>
       </c>
-      <c r="B43" s="57" t="n">
-        <v>102084.9304152285</v>
+      <c r="B43" s="57">
+        <f>F36</f>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -20182,8 +20307,9 @@
           <t>Total Return</t>
         </is>
       </c>
-      <c r="B44" s="57" t="n">
-        <v>5966238.816421503</v>
+      <c r="B44" s="57">
+        <f>B43+B44</f>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -20192,8 +20318,9 @@
           <t>Initial Equity</t>
         </is>
       </c>
-      <c r="B45" s="57" t="n">
-        <v>1955000</v>
+      <c r="B45" s="57">
+        <f>B20</f>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -20202,8 +20329,9 @@
           <t>Equity Multiple</t>
         </is>
       </c>
-      <c r="B46" s="59" t="n">
-        <v>3.051784560829413</v>
+      <c r="B46" s="59">
+        <f>IFERROR(B45/B46,0)</f>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -20212,12 +20340,43 @@
           <t>IRR</t>
         </is>
       </c>
-      <c r="B47" s="56" t="n">
-        <v>0.2483095921905548</v>
+      <c r="B47" s="56">
+        <f>IRR(B49:G49)</f>
+        <v/>
       </c>
     </row>
     <row r="48"/>
-    <row r="49"/>
+    <row r="49">
+      <c r="A49" s="60" t="inlineStr">
+        <is>
+          <t>IRR Cash Flows (Year 0 to Year 5)</t>
+        </is>
+      </c>
+      <c r="B49" s="57">
+        <f>-$B$20</f>
+        <v/>
+      </c>
+      <c r="C49" s="57">
+        <f>B34</f>
+        <v/>
+      </c>
+      <c r="D49" s="57">
+        <f>C34</f>
+        <v/>
+      </c>
+      <c r="E49" s="57">
+        <f>D34</f>
+        <v/>
+      </c>
+      <c r="F49" s="57">
+        <f>E34</f>
+        <v/>
+      </c>
+      <c r="G49" s="57">
+        <f>F34+$B$43</f>
+        <v/>
+      </c>
+    </row>
     <row r="50">
       <c r="A50" s="58" t="inlineStr">
         <is>
@@ -20257,144 +20416,197 @@
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="60" t="n">
+    <row r="52"/>
+    <row r="53">
+      <c r="B53" s="61" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="C53" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="61" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="F53" s="61" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="62" t="n">
         <v>0.055</v>
       </c>
-      <c r="B52" s="61" t="n">
-        <v>0.2721047563746169</v>
-      </c>
-      <c r="C52" s="61" t="n">
-        <v>0.2880719075812196</v>
-      </c>
-      <c r="D52" s="61" t="n">
-        <v>0.2880719075812196</v>
-      </c>
-      <c r="E52" s="61" t="n">
-        <v>0.3032849461413913</v>
-      </c>
-      <c r="F52" s="61" t="n">
-        <v>0.3178196192521103</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="60" t="n">
+      <c r="B54" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*B$53)/$A54)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="C54" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*C$53)/$A54)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="D54" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*D$53)/$A54)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="E54" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*E$53)/$A54)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="F54" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*F$53)/$A54)-$B$42)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="62" t="n">
         <v>0.0575</v>
       </c>
-      <c r="B53" s="61" t="n">
-        <v>0.2582824296655034</v>
-      </c>
-      <c r="C53" s="61" t="n">
-        <v>0.2742332082475913</v>
-      </c>
-      <c r="D53" s="61" t="n">
-        <v>0.2742332082475913</v>
-      </c>
-      <c r="E53" s="61" t="n">
-        <v>0.2894235400893012</v>
-      </c>
-      <c r="F53" s="61" t="n">
-        <v>0.3039304914532881</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="60" t="n">
+      <c r="B55" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*B$53)/$A55)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="C55" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*C$53)/$A55)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="D55" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*D$53)/$A55)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="E55" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*E$53)/$A55)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="F55" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*F$53)/$A55)-$B$42)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="62" t="n">
         <v>0.06</v>
       </c>
-      <c r="B54" s="61" t="n">
-        <v>0.2450556241915656</v>
-      </c>
-      <c r="C54" s="61" t="n">
-        <v>0.2609973815794902</v>
-      </c>
-      <c r="D54" s="61" t="n">
-        <v>0.2609973815794902</v>
-      </c>
-      <c r="E54" s="61" t="n">
-        <v>0.2761718810378718</v>
-      </c>
-      <c r="F54" s="61" t="n">
-        <v>0.2906575807022166</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="60" t="n">
+      <c r="B56" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*B$53)/$A56)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="C56" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*C$53)/$A56)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="D56" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*D$53)/$A56)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="E56" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*E$53)/$A56)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="F56" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*F$53)/$A56)-$B$42)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="62" t="n">
         <v>0.0625</v>
       </c>
-      <c r="B55" s="61" t="n">
-        <v>0.2323699848946241</v>
-      </c>
-      <c r="C55" s="61" t="n">
-        <v>0.2483095921905548</v>
-      </c>
-      <c r="D55" s="61" t="n">
-        <v>0.2483095921905548</v>
-      </c>
-      <c r="E55" s="61" t="n">
-        <v>0.2634746628613108</v>
-      </c>
-      <c r="F55" s="61" t="n">
-        <v>0.2779451207263591</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="60" t="n">
+      <c r="B57" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*B$53)/$A57)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="C57" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*C$53)/$A57)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="D57" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*D$53)/$A57)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="E57" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*E$53)/$A57)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="F57" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*F$53)/$A57)-$B$42)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="62" t="n">
         <v>0.065</v>
       </c>
-      <c r="B56" s="61" t="n">
-        <v>0.22017788947152</v>
-      </c>
-      <c r="C56" s="61" t="n">
-        <v>0.2361218059578299</v>
-      </c>
-      <c r="D56" s="61" t="n">
-        <v>0.2361218059578299</v>
-      </c>
-      <c r="E56" s="61" t="n">
-        <v>0.2512834462014333</v>
-      </c>
-      <c r="F56" s="61" t="n">
-        <v>0.2657442748722254</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="60" t="n">
+      <c r="B58" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*B$53)/$A58)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="C58" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*C$53)/$A58)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="D58" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*D$53)/$A58)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="E58" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*E$53)/$A58)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="F58" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*F$53)/$A58)-$B$42)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="62" t="n">
         <v>0.0675</v>
       </c>
-      <c r="B57" s="61" t="n">
-        <v>0.2084373850784495</v>
-      </c>
-      <c r="C57" s="61" t="n">
-        <v>0.2243917162125861</v>
-      </c>
-      <c r="D57" s="61" t="n">
-        <v>0.2243917162125861</v>
-      </c>
-      <c r="E57" s="61" t="n">
-        <v>0.2395555745201499</v>
-      </c>
-      <c r="F57" s="61" t="n">
-        <v>0.2540120423711922</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="60" t="n">
+      <c r="B59" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*B$53)/$A59)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="C59" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*C$53)/$A59)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="D59" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*D$53)/$A59)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="E59" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*E$53)/$A59)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="F59" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*F$53)/$A59)-$B$42)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="62" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="B58" s="61" t="n">
-        <v>0.197111325171002</v>
-      </c>
-      <c r="C58" s="61" t="n">
-        <v>0.2130818720811583</v>
-      </c>
-      <c r="D58" s="61" t="n">
-        <v>0.2130818720811583</v>
-      </c>
-      <c r="E58" s="61" t="n">
-        <v>0.2282532942369244</v>
-      </c>
-      <c r="F58" s="61" t="n">
-        <v>0.2427103705538361</v>
+      <c r="B60" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*B$53)/$A60)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="C60" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*C$53)/$A60)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="D60" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*D$53)/$A60)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="E60" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*E$53)/$A60)-$B$42)))</f>
+        <v/>
+      </c>
+      <c r="F60" s="56">
+        <f>IRR(CHOOSE(ROW(INDIRECT("1:6")),-$B$20,$B$34,$C$34,$D$34,$E$34,$F$34+((($F$31*F$53)/$A60)-$B$42)))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -20405,6 +20617,18 @@
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B54:F60">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>0.15</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+      <formula>0.10</formula>
+      <formula>0.15</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="2">
+      <formula>0.10</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>